<commit_message>
daily auto push: 2026-09-13 08:15 UTC
</commit_message>
<xml_diff>
--- a/excel/apple2.xlsx
+++ b/excel/apple2.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D4985"/>
+  <dimension ref="A1:D4986"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -89409,16 +89409,16 @@
     <row r="4944">
       <c r="A4944" t="inlineStr">
         <is>
-          <t>2026/12/29</t>
+          <t>2026/09/13</t>
         </is>
       </c>
       <c r="B4944" t="inlineStr">
         <is>
-          <t>火</t>
+          <t>日</t>
         </is>
       </c>
       <c r="C4944" t="n">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="D4944" t="n">
         <v>201</v>
@@ -89436,7 +89436,7 @@
         </is>
       </c>
       <c r="C4945" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D4945" t="n">
         <v>201</v>
@@ -89454,7 +89454,7 @@
         </is>
       </c>
       <c r="C4946" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D4946" t="n">
         <v>201</v>
@@ -89472,7 +89472,7 @@
         </is>
       </c>
       <c r="C4947" t="n">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="D4947" t="n">
         <v>201</v>
@@ -89481,16 +89481,16 @@
     <row r="4948">
       <c r="A4948" t="inlineStr">
         <is>
-          <t>2026/12/30</t>
+          <t>2026/12/29</t>
         </is>
       </c>
       <c r="B4948" t="inlineStr">
         <is>
-          <t>水</t>
+          <t>火</t>
         </is>
       </c>
       <c r="C4948" t="n">
-        <v>2</v>
+        <v>23</v>
       </c>
       <c r="D4948" t="n">
         <v>201</v>
@@ -89508,7 +89508,7 @@
         </is>
       </c>
       <c r="C4949" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D4949" t="n">
         <v>201</v>
@@ -89526,7 +89526,7 @@
         </is>
       </c>
       <c r="C4950" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D4950" t="n">
         <v>201</v>
@@ -89544,7 +89544,7 @@
         </is>
       </c>
       <c r="C4951" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="D4951" t="n">
         <v>201</v>
@@ -89562,7 +89562,7 @@
         </is>
       </c>
       <c r="C4952" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D4952" t="n">
         <v>201</v>
@@ -89580,7 +89580,7 @@
         </is>
       </c>
       <c r="C4953" t="n">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="D4953" t="n">
         <v>201</v>
@@ -89589,16 +89589,16 @@
     <row r="4954">
       <c r="A4954" t="inlineStr">
         <is>
-          <t>2026/12/31</t>
+          <t>2026/12/30</t>
         </is>
       </c>
       <c r="B4954" t="inlineStr">
         <is>
-          <t>木</t>
+          <t>水</t>
         </is>
       </c>
       <c r="C4954" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D4954" t="n">
         <v>201</v>
@@ -89616,7 +89616,7 @@
         </is>
       </c>
       <c r="C4955" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="D4955" t="n">
         <v>201</v>
@@ -89634,7 +89634,7 @@
         </is>
       </c>
       <c r="C4956" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="D4956" t="n">
         <v>201</v>
@@ -89652,7 +89652,7 @@
         </is>
       </c>
       <c r="C4957" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="D4957" t="n">
         <v>201</v>
@@ -89670,7 +89670,7 @@
         </is>
       </c>
       <c r="C4958" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="D4958" t="n">
         <v>201</v>
@@ -89688,7 +89688,7 @@
         </is>
       </c>
       <c r="C4959" t="n">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="D4959" t="n">
         <v>201</v>
@@ -89697,16 +89697,16 @@
     <row r="4960">
       <c r="A4960" t="inlineStr">
         <is>
-          <t>2027/01/01</t>
+          <t>2026/12/31</t>
         </is>
       </c>
       <c r="B4960" t="inlineStr">
         <is>
-          <t>金</t>
+          <t>木</t>
         </is>
       </c>
       <c r="C4960" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D4960" t="n">
         <v>201</v>
@@ -89724,7 +89724,7 @@
         </is>
       </c>
       <c r="C4961" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D4961" t="n">
         <v>201</v>
@@ -89742,7 +89742,7 @@
         </is>
       </c>
       <c r="C4962" t="n">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="D4962" t="n">
         <v>201</v>
@@ -89760,7 +89760,7 @@
         </is>
       </c>
       <c r="C4963" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D4963" t="n">
         <v>201</v>
@@ -89778,7 +89778,7 @@
         </is>
       </c>
       <c r="C4964" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D4964" t="n">
         <v>201</v>
@@ -89787,16 +89787,16 @@
     <row r="4965">
       <c r="A4965" t="inlineStr">
         <is>
-          <t>2027/01/02</t>
+          <t>2027/01/01</t>
         </is>
       </c>
       <c r="B4965" t="inlineStr">
         <is>
-          <t>土</t>
+          <t>金</t>
         </is>
       </c>
       <c r="C4965" t="n">
-        <v>1</v>
+        <v>19</v>
       </c>
       <c r="D4965" t="n">
         <v>201</v>
@@ -89814,7 +89814,7 @@
         </is>
       </c>
       <c r="C4966" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D4966" t="n">
         <v>201</v>
@@ -89832,7 +89832,7 @@
         </is>
       </c>
       <c r="C4967" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D4967" t="n">
         <v>201</v>
@@ -89850,7 +89850,7 @@
         </is>
       </c>
       <c r="C4968" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="D4968" t="n">
         <v>201</v>
@@ -89868,7 +89868,7 @@
         </is>
       </c>
       <c r="C4969" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D4969" t="n">
         <v>201</v>
@@ -89886,7 +89886,7 @@
         </is>
       </c>
       <c r="C4970" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D4970" t="n">
         <v>201</v>
@@ -89904,7 +89904,7 @@
         </is>
       </c>
       <c r="C4971" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="D4971" t="n">
         <v>201</v>
@@ -89913,16 +89913,16 @@
     <row r="4972">
       <c r="A4972" t="inlineStr">
         <is>
-          <t>2027/01/03</t>
+          <t>2027/01/02</t>
         </is>
       </c>
       <c r="B4972" t="inlineStr">
         <is>
-          <t>日</t>
+          <t>土</t>
         </is>
       </c>
       <c r="C4972" t="n">
-        <v>1</v>
+        <v>22</v>
       </c>
       <c r="D4972" t="n">
         <v>201</v>
@@ -89940,7 +89940,7 @@
         </is>
       </c>
       <c r="C4973" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D4973" t="n">
         <v>201</v>
@@ -89958,7 +89958,7 @@
         </is>
       </c>
       <c r="C4974" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D4974" t="n">
         <v>201</v>
@@ -89976,7 +89976,7 @@
         </is>
       </c>
       <c r="C4975" t="n">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="D4975" t="n">
         <v>201</v>
@@ -89994,7 +89994,7 @@
         </is>
       </c>
       <c r="C4976" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D4976" t="n">
         <v>201</v>
@@ -90012,7 +90012,7 @@
         </is>
       </c>
       <c r="C4977" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D4977" t="n">
         <v>201</v>
@@ -90030,7 +90030,7 @@
         </is>
       </c>
       <c r="C4978" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="D4978" t="n">
         <v>201</v>
@@ -90039,16 +90039,16 @@
     <row r="4979">
       <c r="A4979" t="inlineStr">
         <is>
-          <t>2027/01/04</t>
+          <t>2027/01/03</t>
         </is>
       </c>
       <c r="B4979" t="inlineStr">
         <is>
-          <t>月</t>
+          <t>日</t>
         </is>
       </c>
       <c r="C4979" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D4979" t="n">
         <v>201</v>
@@ -90066,7 +90066,7 @@
         </is>
       </c>
       <c r="C4980" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D4980" t="n">
         <v>201</v>
@@ -90084,7 +90084,7 @@
         </is>
       </c>
       <c r="C4981" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D4981" t="n">
         <v>201</v>
@@ -90102,7 +90102,7 @@
         </is>
       </c>
       <c r="C4982" t="n">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="D4982" t="n">
         <v>201</v>
@@ -90120,7 +90120,7 @@
         </is>
       </c>
       <c r="C4983" t="n">
-        <v>22</v>
+        <v>13</v>
       </c>
       <c r="D4983" t="n">
         <v>201</v>
@@ -90129,16 +90129,16 @@
     <row r="4984">
       <c r="A4984" t="inlineStr">
         <is>
-          <t>2027/01/05</t>
+          <t>2027/01/04</t>
         </is>
       </c>
       <c r="B4984" t="inlineStr">
         <is>
-          <t>火</t>
+          <t>月</t>
         </is>
       </c>
       <c r="C4984" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D4984" t="n">
         <v>201</v>
@@ -90156,9 +90156,27 @@
         </is>
       </c>
       <c r="C4985" t="n">
+        <v>2</v>
+      </c>
+      <c r="D4985" t="n">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="4986">
+      <c r="A4986" t="inlineStr">
+        <is>
+          <t>2027/01/05</t>
+        </is>
+      </c>
+      <c r="B4986" t="inlineStr">
+        <is>
+          <t>火</t>
+        </is>
+      </c>
+      <c r="C4986" t="n">
         <v>7</v>
       </c>
-      <c r="D4985" t="n">
+      <c r="D4986" t="n">
         <v>201</v>
       </c>
     </row>

</xml_diff>

<commit_message>
daily auto push: 2026-09-16 07:37 UTC
</commit_message>
<xml_diff>
--- a/excel/apple2.xlsx
+++ b/excel/apple2.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D5006"/>
+  <dimension ref="A1:D5007"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -89787,16 +89787,16 @@
     <row r="4965">
       <c r="A4965" t="inlineStr">
         <is>
-          <t>2026/12/29</t>
+          <t>2026/09/16</t>
         </is>
       </c>
       <c r="B4965" t="inlineStr">
         <is>
-          <t>火</t>
+          <t>水</t>
         </is>
       </c>
       <c r="C4965" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D4965" t="n">
         <v>201</v>
@@ -89814,7 +89814,7 @@
         </is>
       </c>
       <c r="C4966" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D4966" t="n">
         <v>201</v>
@@ -89832,7 +89832,7 @@
         </is>
       </c>
       <c r="C4967" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D4967" t="n">
         <v>201</v>
@@ -89850,7 +89850,7 @@
         </is>
       </c>
       <c r="C4968" t="n">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="D4968" t="n">
         <v>201</v>
@@ -89859,16 +89859,16 @@
     <row r="4969">
       <c r="A4969" t="inlineStr">
         <is>
-          <t>2026/12/30</t>
+          <t>2026/12/29</t>
         </is>
       </c>
       <c r="B4969" t="inlineStr">
         <is>
-          <t>水</t>
+          <t>火</t>
         </is>
       </c>
       <c r="C4969" t="n">
-        <v>2</v>
+        <v>23</v>
       </c>
       <c r="D4969" t="n">
         <v>201</v>
@@ -89886,7 +89886,7 @@
         </is>
       </c>
       <c r="C4970" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D4970" t="n">
         <v>201</v>
@@ -89904,7 +89904,7 @@
         </is>
       </c>
       <c r="C4971" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D4971" t="n">
         <v>201</v>
@@ -89922,7 +89922,7 @@
         </is>
       </c>
       <c r="C4972" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="D4972" t="n">
         <v>201</v>
@@ -89940,7 +89940,7 @@
         </is>
       </c>
       <c r="C4973" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D4973" t="n">
         <v>201</v>
@@ -89958,7 +89958,7 @@
         </is>
       </c>
       <c r="C4974" t="n">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="D4974" t="n">
         <v>201</v>
@@ -89967,16 +89967,16 @@
     <row r="4975">
       <c r="A4975" t="inlineStr">
         <is>
-          <t>2026/12/31</t>
+          <t>2026/12/30</t>
         </is>
       </c>
       <c r="B4975" t="inlineStr">
         <is>
-          <t>木</t>
+          <t>水</t>
         </is>
       </c>
       <c r="C4975" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D4975" t="n">
         <v>201</v>
@@ -89994,7 +89994,7 @@
         </is>
       </c>
       <c r="C4976" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="D4976" t="n">
         <v>201</v>
@@ -90012,7 +90012,7 @@
         </is>
       </c>
       <c r="C4977" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="D4977" t="n">
         <v>201</v>
@@ -90030,7 +90030,7 @@
         </is>
       </c>
       <c r="C4978" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="D4978" t="n">
         <v>201</v>
@@ -90048,7 +90048,7 @@
         </is>
       </c>
       <c r="C4979" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="D4979" t="n">
         <v>201</v>
@@ -90066,7 +90066,7 @@
         </is>
       </c>
       <c r="C4980" t="n">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="D4980" t="n">
         <v>201</v>
@@ -90075,16 +90075,16 @@
     <row r="4981">
       <c r="A4981" t="inlineStr">
         <is>
-          <t>2027/01/01</t>
+          <t>2026/12/31</t>
         </is>
       </c>
       <c r="B4981" t="inlineStr">
         <is>
-          <t>金</t>
+          <t>木</t>
         </is>
       </c>
       <c r="C4981" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D4981" t="n">
         <v>201</v>
@@ -90102,7 +90102,7 @@
         </is>
       </c>
       <c r="C4982" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D4982" t="n">
         <v>201</v>
@@ -90120,7 +90120,7 @@
         </is>
       </c>
       <c r="C4983" t="n">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="D4983" t="n">
         <v>201</v>
@@ -90138,7 +90138,7 @@
         </is>
       </c>
       <c r="C4984" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D4984" t="n">
         <v>201</v>
@@ -90156,7 +90156,7 @@
         </is>
       </c>
       <c r="C4985" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D4985" t="n">
         <v>201</v>
@@ -90165,16 +90165,16 @@
     <row r="4986">
       <c r="A4986" t="inlineStr">
         <is>
-          <t>2027/01/02</t>
+          <t>2027/01/01</t>
         </is>
       </c>
       <c r="B4986" t="inlineStr">
         <is>
-          <t>土</t>
+          <t>金</t>
         </is>
       </c>
       <c r="C4986" t="n">
-        <v>1</v>
+        <v>19</v>
       </c>
       <c r="D4986" t="n">
         <v>201</v>
@@ -90192,7 +90192,7 @@
         </is>
       </c>
       <c r="C4987" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D4987" t="n">
         <v>201</v>
@@ -90210,7 +90210,7 @@
         </is>
       </c>
       <c r="C4988" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D4988" t="n">
         <v>201</v>
@@ -90228,7 +90228,7 @@
         </is>
       </c>
       <c r="C4989" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="D4989" t="n">
         <v>201</v>
@@ -90246,7 +90246,7 @@
         </is>
       </c>
       <c r="C4990" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D4990" t="n">
         <v>201</v>
@@ -90264,7 +90264,7 @@
         </is>
       </c>
       <c r="C4991" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D4991" t="n">
         <v>201</v>
@@ -90282,7 +90282,7 @@
         </is>
       </c>
       <c r="C4992" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="D4992" t="n">
         <v>201</v>
@@ -90291,16 +90291,16 @@
     <row r="4993">
       <c r="A4993" t="inlineStr">
         <is>
-          <t>2027/01/03</t>
+          <t>2027/01/02</t>
         </is>
       </c>
       <c r="B4993" t="inlineStr">
         <is>
-          <t>日</t>
+          <t>土</t>
         </is>
       </c>
       <c r="C4993" t="n">
-        <v>1</v>
+        <v>22</v>
       </c>
       <c r="D4993" t="n">
         <v>201</v>
@@ -90318,7 +90318,7 @@
         </is>
       </c>
       <c r="C4994" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D4994" t="n">
         <v>201</v>
@@ -90336,7 +90336,7 @@
         </is>
       </c>
       <c r="C4995" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D4995" t="n">
         <v>201</v>
@@ -90354,7 +90354,7 @@
         </is>
       </c>
       <c r="C4996" t="n">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="D4996" t="n">
         <v>201</v>
@@ -90372,7 +90372,7 @@
         </is>
       </c>
       <c r="C4997" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D4997" t="n">
         <v>201</v>
@@ -90390,7 +90390,7 @@
         </is>
       </c>
       <c r="C4998" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D4998" t="n">
         <v>201</v>
@@ -90408,7 +90408,7 @@
         </is>
       </c>
       <c r="C4999" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="D4999" t="n">
         <v>201</v>
@@ -90417,16 +90417,16 @@
     <row r="5000">
       <c r="A5000" t="inlineStr">
         <is>
-          <t>2027/01/04</t>
+          <t>2027/01/03</t>
         </is>
       </c>
       <c r="B5000" t="inlineStr">
         <is>
-          <t>月</t>
+          <t>日</t>
         </is>
       </c>
       <c r="C5000" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D5000" t="n">
         <v>201</v>
@@ -90444,7 +90444,7 @@
         </is>
       </c>
       <c r="C5001" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D5001" t="n">
         <v>201</v>
@@ -90462,7 +90462,7 @@
         </is>
       </c>
       <c r="C5002" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D5002" t="n">
         <v>201</v>
@@ -90480,7 +90480,7 @@
         </is>
       </c>
       <c r="C5003" t="n">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="D5003" t="n">
         <v>201</v>
@@ -90498,7 +90498,7 @@
         </is>
       </c>
       <c r="C5004" t="n">
-        <v>22</v>
+        <v>13</v>
       </c>
       <c r="D5004" t="n">
         <v>201</v>
@@ -90507,16 +90507,16 @@
     <row r="5005">
       <c r="A5005" t="inlineStr">
         <is>
-          <t>2027/01/05</t>
+          <t>2027/01/04</t>
         </is>
       </c>
       <c r="B5005" t="inlineStr">
         <is>
-          <t>火</t>
+          <t>月</t>
         </is>
       </c>
       <c r="C5005" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D5005" t="n">
         <v>201</v>
@@ -90534,9 +90534,27 @@
         </is>
       </c>
       <c r="C5006" t="n">
+        <v>2</v>
+      </c>
+      <c r="D5006" t="n">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="5007">
+      <c r="A5007" t="inlineStr">
+        <is>
+          <t>2027/01/05</t>
+        </is>
+      </c>
+      <c r="B5007" t="inlineStr">
+        <is>
+          <t>火</t>
+        </is>
+      </c>
+      <c r="C5007" t="n">
         <v>7</v>
       </c>
-      <c r="D5006" t="n">
+      <c r="D5007" t="n">
         <v>201</v>
       </c>
     </row>

</xml_diff>

<commit_message>
daily auto push: 2026-09-18 07:22 UTC
</commit_message>
<xml_diff>
--- a/excel/apple2.xlsx
+++ b/excel/apple2.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D5020"/>
+  <dimension ref="A1:D5021"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -90039,16 +90039,16 @@
     <row r="4979">
       <c r="A4979" t="inlineStr">
         <is>
-          <t>2026/12/29</t>
+          <t>2026/09/18</t>
         </is>
       </c>
       <c r="B4979" t="inlineStr">
         <is>
-          <t>火</t>
+          <t>金</t>
         </is>
       </c>
       <c r="C4979" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D4979" t="n">
         <v>201</v>
@@ -90066,7 +90066,7 @@
         </is>
       </c>
       <c r="C4980" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D4980" t="n">
         <v>201</v>
@@ -90084,7 +90084,7 @@
         </is>
       </c>
       <c r="C4981" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D4981" t="n">
         <v>201</v>
@@ -90102,7 +90102,7 @@
         </is>
       </c>
       <c r="C4982" t="n">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="D4982" t="n">
         <v>201</v>
@@ -90111,16 +90111,16 @@
     <row r="4983">
       <c r="A4983" t="inlineStr">
         <is>
-          <t>2026/12/30</t>
+          <t>2026/12/29</t>
         </is>
       </c>
       <c r="B4983" t="inlineStr">
         <is>
-          <t>水</t>
+          <t>火</t>
         </is>
       </c>
       <c r="C4983" t="n">
-        <v>2</v>
+        <v>23</v>
       </c>
       <c r="D4983" t="n">
         <v>201</v>
@@ -90138,7 +90138,7 @@
         </is>
       </c>
       <c r="C4984" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D4984" t="n">
         <v>201</v>
@@ -90156,7 +90156,7 @@
         </is>
       </c>
       <c r="C4985" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D4985" t="n">
         <v>201</v>
@@ -90174,7 +90174,7 @@
         </is>
       </c>
       <c r="C4986" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="D4986" t="n">
         <v>201</v>
@@ -90192,7 +90192,7 @@
         </is>
       </c>
       <c r="C4987" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D4987" t="n">
         <v>201</v>
@@ -90210,7 +90210,7 @@
         </is>
       </c>
       <c r="C4988" t="n">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="D4988" t="n">
         <v>201</v>
@@ -90219,16 +90219,16 @@
     <row r="4989">
       <c r="A4989" t="inlineStr">
         <is>
-          <t>2026/12/31</t>
+          <t>2026/12/30</t>
         </is>
       </c>
       <c r="B4989" t="inlineStr">
         <is>
-          <t>木</t>
+          <t>水</t>
         </is>
       </c>
       <c r="C4989" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D4989" t="n">
         <v>201</v>
@@ -90246,7 +90246,7 @@
         </is>
       </c>
       <c r="C4990" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="D4990" t="n">
         <v>201</v>
@@ -90264,7 +90264,7 @@
         </is>
       </c>
       <c r="C4991" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="D4991" t="n">
         <v>201</v>
@@ -90282,7 +90282,7 @@
         </is>
       </c>
       <c r="C4992" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="D4992" t="n">
         <v>201</v>
@@ -90300,7 +90300,7 @@
         </is>
       </c>
       <c r="C4993" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="D4993" t="n">
         <v>201</v>
@@ -90318,7 +90318,7 @@
         </is>
       </c>
       <c r="C4994" t="n">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="D4994" t="n">
         <v>201</v>
@@ -90327,16 +90327,16 @@
     <row r="4995">
       <c r="A4995" t="inlineStr">
         <is>
-          <t>2027/01/01</t>
+          <t>2026/12/31</t>
         </is>
       </c>
       <c r="B4995" t="inlineStr">
         <is>
-          <t>金</t>
+          <t>木</t>
         </is>
       </c>
       <c r="C4995" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D4995" t="n">
         <v>201</v>
@@ -90354,7 +90354,7 @@
         </is>
       </c>
       <c r="C4996" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D4996" t="n">
         <v>201</v>
@@ -90372,7 +90372,7 @@
         </is>
       </c>
       <c r="C4997" t="n">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="D4997" t="n">
         <v>201</v>
@@ -90390,7 +90390,7 @@
         </is>
       </c>
       <c r="C4998" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D4998" t="n">
         <v>201</v>
@@ -90408,7 +90408,7 @@
         </is>
       </c>
       <c r="C4999" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D4999" t="n">
         <v>201</v>
@@ -90417,16 +90417,16 @@
     <row r="5000">
       <c r="A5000" t="inlineStr">
         <is>
-          <t>2027/01/02</t>
+          <t>2027/01/01</t>
         </is>
       </c>
       <c r="B5000" t="inlineStr">
         <is>
-          <t>土</t>
+          <t>金</t>
         </is>
       </c>
       <c r="C5000" t="n">
-        <v>1</v>
+        <v>19</v>
       </c>
       <c r="D5000" t="n">
         <v>201</v>
@@ -90444,7 +90444,7 @@
         </is>
       </c>
       <c r="C5001" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D5001" t="n">
         <v>201</v>
@@ -90462,7 +90462,7 @@
         </is>
       </c>
       <c r="C5002" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D5002" t="n">
         <v>201</v>
@@ -90480,7 +90480,7 @@
         </is>
       </c>
       <c r="C5003" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="D5003" t="n">
         <v>201</v>
@@ -90498,7 +90498,7 @@
         </is>
       </c>
       <c r="C5004" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D5004" t="n">
         <v>201</v>
@@ -90516,7 +90516,7 @@
         </is>
       </c>
       <c r="C5005" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D5005" t="n">
         <v>201</v>
@@ -90534,7 +90534,7 @@
         </is>
       </c>
       <c r="C5006" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="D5006" t="n">
         <v>201</v>
@@ -90543,16 +90543,16 @@
     <row r="5007">
       <c r="A5007" t="inlineStr">
         <is>
-          <t>2027/01/03</t>
+          <t>2027/01/02</t>
         </is>
       </c>
       <c r="B5007" t="inlineStr">
         <is>
-          <t>日</t>
+          <t>土</t>
         </is>
       </c>
       <c r="C5007" t="n">
-        <v>1</v>
+        <v>22</v>
       </c>
       <c r="D5007" t="n">
         <v>201</v>
@@ -90570,7 +90570,7 @@
         </is>
       </c>
       <c r="C5008" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D5008" t="n">
         <v>201</v>
@@ -90588,7 +90588,7 @@
         </is>
       </c>
       <c r="C5009" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D5009" t="n">
         <v>201</v>
@@ -90606,7 +90606,7 @@
         </is>
       </c>
       <c r="C5010" t="n">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="D5010" t="n">
         <v>201</v>
@@ -90624,7 +90624,7 @@
         </is>
       </c>
       <c r="C5011" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D5011" t="n">
         <v>201</v>
@@ -90642,7 +90642,7 @@
         </is>
       </c>
       <c r="C5012" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D5012" t="n">
         <v>201</v>
@@ -90660,7 +90660,7 @@
         </is>
       </c>
       <c r="C5013" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="D5013" t="n">
         <v>201</v>
@@ -90669,16 +90669,16 @@
     <row r="5014">
       <c r="A5014" t="inlineStr">
         <is>
-          <t>2027/01/04</t>
+          <t>2027/01/03</t>
         </is>
       </c>
       <c r="B5014" t="inlineStr">
         <is>
-          <t>月</t>
+          <t>日</t>
         </is>
       </c>
       <c r="C5014" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D5014" t="n">
         <v>201</v>
@@ -90696,7 +90696,7 @@
         </is>
       </c>
       <c r="C5015" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D5015" t="n">
         <v>201</v>
@@ -90714,7 +90714,7 @@
         </is>
       </c>
       <c r="C5016" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D5016" t="n">
         <v>201</v>
@@ -90732,7 +90732,7 @@
         </is>
       </c>
       <c r="C5017" t="n">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="D5017" t="n">
         <v>201</v>
@@ -90750,7 +90750,7 @@
         </is>
       </c>
       <c r="C5018" t="n">
-        <v>22</v>
+        <v>13</v>
       </c>
       <c r="D5018" t="n">
         <v>201</v>
@@ -90759,16 +90759,16 @@
     <row r="5019">
       <c r="A5019" t="inlineStr">
         <is>
-          <t>2027/01/05</t>
+          <t>2027/01/04</t>
         </is>
       </c>
       <c r="B5019" t="inlineStr">
         <is>
-          <t>火</t>
+          <t>月</t>
         </is>
       </c>
       <c r="C5019" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D5019" t="n">
         <v>201</v>
@@ -90786,9 +90786,27 @@
         </is>
       </c>
       <c r="C5020" t="n">
+        <v>2</v>
+      </c>
+      <c r="D5020" t="n">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="5021">
+      <c r="A5021" t="inlineStr">
+        <is>
+          <t>2027/01/05</t>
+        </is>
+      </c>
+      <c r="B5021" t="inlineStr">
+        <is>
+          <t>火</t>
+        </is>
+      </c>
+      <c r="C5021" t="n">
         <v>7</v>
       </c>
-      <c r="D5020" t="n">
+      <c r="D5021" t="n">
         <v>201</v>
       </c>
     </row>

</xml_diff>

<commit_message>
daily auto push: 2026-09-19 20:33 UTC
</commit_message>
<xml_diff>
--- a/excel/apple2.xlsx
+++ b/excel/apple2.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D5031"/>
+  <dimension ref="A1:D5032"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -90237,16 +90237,16 @@
     <row r="4990">
       <c r="A4990" t="inlineStr">
         <is>
-          <t>2026/12/29</t>
+          <t>2026/09/20</t>
         </is>
       </c>
       <c r="B4990" t="inlineStr">
         <is>
-          <t>火</t>
+          <t>日</t>
         </is>
       </c>
       <c r="C4990" t="n">
-        <v>13</v>
+        <v>2</v>
       </c>
       <c r="D4990" t="n">
         <v>201</v>
@@ -90264,7 +90264,7 @@
         </is>
       </c>
       <c r="C4991" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D4991" t="n">
         <v>201</v>
@@ -90282,7 +90282,7 @@
         </is>
       </c>
       <c r="C4992" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D4992" t="n">
         <v>201</v>
@@ -90300,7 +90300,7 @@
         </is>
       </c>
       <c r="C4993" t="n">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="D4993" t="n">
         <v>201</v>
@@ -90309,16 +90309,16 @@
     <row r="4994">
       <c r="A4994" t="inlineStr">
         <is>
-          <t>2026/12/30</t>
+          <t>2026/12/29</t>
         </is>
       </c>
       <c r="B4994" t="inlineStr">
         <is>
-          <t>水</t>
+          <t>火</t>
         </is>
       </c>
       <c r="C4994" t="n">
-        <v>2</v>
+        <v>23</v>
       </c>
       <c r="D4994" t="n">
         <v>201</v>
@@ -90336,7 +90336,7 @@
         </is>
       </c>
       <c r="C4995" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D4995" t="n">
         <v>201</v>
@@ -90354,7 +90354,7 @@
         </is>
       </c>
       <c r="C4996" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D4996" t="n">
         <v>201</v>
@@ -90372,7 +90372,7 @@
         </is>
       </c>
       <c r="C4997" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="D4997" t="n">
         <v>201</v>
@@ -90390,7 +90390,7 @@
         </is>
       </c>
       <c r="C4998" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D4998" t="n">
         <v>201</v>
@@ -90408,7 +90408,7 @@
         </is>
       </c>
       <c r="C4999" t="n">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="D4999" t="n">
         <v>201</v>
@@ -90417,16 +90417,16 @@
     <row r="5000">
       <c r="A5000" t="inlineStr">
         <is>
-          <t>2026/12/31</t>
+          <t>2026/12/30</t>
         </is>
       </c>
       <c r="B5000" t="inlineStr">
         <is>
-          <t>木</t>
+          <t>水</t>
         </is>
       </c>
       <c r="C5000" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D5000" t="n">
         <v>201</v>
@@ -90444,7 +90444,7 @@
         </is>
       </c>
       <c r="C5001" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="D5001" t="n">
         <v>201</v>
@@ -90462,7 +90462,7 @@
         </is>
       </c>
       <c r="C5002" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="D5002" t="n">
         <v>201</v>
@@ -90480,7 +90480,7 @@
         </is>
       </c>
       <c r="C5003" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="D5003" t="n">
         <v>201</v>
@@ -90498,7 +90498,7 @@
         </is>
       </c>
       <c r="C5004" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="D5004" t="n">
         <v>201</v>
@@ -90516,7 +90516,7 @@
         </is>
       </c>
       <c r="C5005" t="n">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="D5005" t="n">
         <v>201</v>
@@ -90525,16 +90525,16 @@
     <row r="5006">
       <c r="A5006" t="inlineStr">
         <is>
-          <t>2027/01/01</t>
+          <t>2026/12/31</t>
         </is>
       </c>
       <c r="B5006" t="inlineStr">
         <is>
-          <t>金</t>
+          <t>木</t>
         </is>
       </c>
       <c r="C5006" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D5006" t="n">
         <v>201</v>
@@ -90552,7 +90552,7 @@
         </is>
       </c>
       <c r="C5007" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D5007" t="n">
         <v>201</v>
@@ -90570,7 +90570,7 @@
         </is>
       </c>
       <c r="C5008" t="n">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="D5008" t="n">
         <v>201</v>
@@ -90588,7 +90588,7 @@
         </is>
       </c>
       <c r="C5009" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D5009" t="n">
         <v>201</v>
@@ -90606,7 +90606,7 @@
         </is>
       </c>
       <c r="C5010" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D5010" t="n">
         <v>201</v>
@@ -90615,16 +90615,16 @@
     <row r="5011">
       <c r="A5011" t="inlineStr">
         <is>
-          <t>2027/01/02</t>
+          <t>2027/01/01</t>
         </is>
       </c>
       <c r="B5011" t="inlineStr">
         <is>
-          <t>土</t>
+          <t>金</t>
         </is>
       </c>
       <c r="C5011" t="n">
-        <v>1</v>
+        <v>19</v>
       </c>
       <c r="D5011" t="n">
         <v>201</v>
@@ -90642,7 +90642,7 @@
         </is>
       </c>
       <c r="C5012" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D5012" t="n">
         <v>201</v>
@@ -90660,7 +90660,7 @@
         </is>
       </c>
       <c r="C5013" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D5013" t="n">
         <v>201</v>
@@ -90678,7 +90678,7 @@
         </is>
       </c>
       <c r="C5014" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="D5014" t="n">
         <v>201</v>
@@ -90696,7 +90696,7 @@
         </is>
       </c>
       <c r="C5015" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D5015" t="n">
         <v>201</v>
@@ -90714,7 +90714,7 @@
         </is>
       </c>
       <c r="C5016" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D5016" t="n">
         <v>201</v>
@@ -90732,7 +90732,7 @@
         </is>
       </c>
       <c r="C5017" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="D5017" t="n">
         <v>201</v>
@@ -90741,16 +90741,16 @@
     <row r="5018">
       <c r="A5018" t="inlineStr">
         <is>
-          <t>2027/01/03</t>
+          <t>2027/01/02</t>
         </is>
       </c>
       <c r="B5018" t="inlineStr">
         <is>
-          <t>日</t>
+          <t>土</t>
         </is>
       </c>
       <c r="C5018" t="n">
-        <v>1</v>
+        <v>22</v>
       </c>
       <c r="D5018" t="n">
         <v>201</v>
@@ -90768,7 +90768,7 @@
         </is>
       </c>
       <c r="C5019" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D5019" t="n">
         <v>201</v>
@@ -90786,7 +90786,7 @@
         </is>
       </c>
       <c r="C5020" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D5020" t="n">
         <v>201</v>
@@ -90804,7 +90804,7 @@
         </is>
       </c>
       <c r="C5021" t="n">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="D5021" t="n">
         <v>201</v>
@@ -90822,7 +90822,7 @@
         </is>
       </c>
       <c r="C5022" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D5022" t="n">
         <v>201</v>
@@ -90840,7 +90840,7 @@
         </is>
       </c>
       <c r="C5023" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D5023" t="n">
         <v>201</v>
@@ -90858,7 +90858,7 @@
         </is>
       </c>
       <c r="C5024" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="D5024" t="n">
         <v>201</v>
@@ -90867,16 +90867,16 @@
     <row r="5025">
       <c r="A5025" t="inlineStr">
         <is>
-          <t>2027/01/04</t>
+          <t>2027/01/03</t>
         </is>
       </c>
       <c r="B5025" t="inlineStr">
         <is>
-          <t>月</t>
+          <t>日</t>
         </is>
       </c>
       <c r="C5025" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D5025" t="n">
         <v>201</v>
@@ -90894,7 +90894,7 @@
         </is>
       </c>
       <c r="C5026" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D5026" t="n">
         <v>201</v>
@@ -90912,7 +90912,7 @@
         </is>
       </c>
       <c r="C5027" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D5027" t="n">
         <v>201</v>
@@ -90930,7 +90930,7 @@
         </is>
       </c>
       <c r="C5028" t="n">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="D5028" t="n">
         <v>201</v>
@@ -90948,7 +90948,7 @@
         </is>
       </c>
       <c r="C5029" t="n">
-        <v>22</v>
+        <v>13</v>
       </c>
       <c r="D5029" t="n">
         <v>201</v>
@@ -90957,16 +90957,16 @@
     <row r="5030">
       <c r="A5030" t="inlineStr">
         <is>
-          <t>2027/01/05</t>
+          <t>2027/01/04</t>
         </is>
       </c>
       <c r="B5030" t="inlineStr">
         <is>
-          <t>火</t>
+          <t>月</t>
         </is>
       </c>
       <c r="C5030" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D5030" t="n">
         <v>201</v>
@@ -90984,9 +90984,27 @@
         </is>
       </c>
       <c r="C5031" t="n">
+        <v>2</v>
+      </c>
+      <c r="D5031" t="n">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="5032">
+      <c r="A5032" t="inlineStr">
+        <is>
+          <t>2027/01/05</t>
+        </is>
+      </c>
+      <c r="B5032" t="inlineStr">
+        <is>
+          <t>火</t>
+        </is>
+      </c>
+      <c r="C5032" t="n">
         <v>7</v>
       </c>
-      <c r="D5031" t="n">
+      <c r="D5032" t="n">
         <v>201</v>
       </c>
     </row>

</xml_diff>

<commit_message>
daily auto push: 2026-09-20 16:46 UTC
</commit_message>
<xml_diff>
--- a/excel/apple2.xlsx
+++ b/excel/apple2.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D5037"/>
+  <dimension ref="A1:D5038"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -90345,16 +90345,16 @@
     <row r="4996">
       <c r="A4996" t="inlineStr">
         <is>
-          <t>2026/12/29</t>
+          <t>2026/09/20</t>
         </is>
       </c>
       <c r="B4996" t="inlineStr">
         <is>
-          <t>火</t>
+          <t>日</t>
         </is>
       </c>
       <c r="C4996" t="n">
-        <v>13</v>
+        <v>23</v>
       </c>
       <c r="D4996" t="n">
         <v>201</v>
@@ -90372,7 +90372,7 @@
         </is>
       </c>
       <c r="C4997" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D4997" t="n">
         <v>201</v>
@@ -90390,7 +90390,7 @@
         </is>
       </c>
       <c r="C4998" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D4998" t="n">
         <v>201</v>
@@ -90408,7 +90408,7 @@
         </is>
       </c>
       <c r="C4999" t="n">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="D4999" t="n">
         <v>201</v>
@@ -90417,16 +90417,16 @@
     <row r="5000">
       <c r="A5000" t="inlineStr">
         <is>
-          <t>2026/12/30</t>
+          <t>2026/12/29</t>
         </is>
       </c>
       <c r="B5000" t="inlineStr">
         <is>
-          <t>水</t>
+          <t>火</t>
         </is>
       </c>
       <c r="C5000" t="n">
-        <v>2</v>
+        <v>23</v>
       </c>
       <c r="D5000" t="n">
         <v>201</v>
@@ -90444,7 +90444,7 @@
         </is>
       </c>
       <c r="C5001" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D5001" t="n">
         <v>201</v>
@@ -90462,7 +90462,7 @@
         </is>
       </c>
       <c r="C5002" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D5002" t="n">
         <v>201</v>
@@ -90480,7 +90480,7 @@
         </is>
       </c>
       <c r="C5003" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="D5003" t="n">
         <v>201</v>
@@ -90498,7 +90498,7 @@
         </is>
       </c>
       <c r="C5004" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D5004" t="n">
         <v>201</v>
@@ -90516,7 +90516,7 @@
         </is>
       </c>
       <c r="C5005" t="n">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="D5005" t="n">
         <v>201</v>
@@ -90525,16 +90525,16 @@
     <row r="5006">
       <c r="A5006" t="inlineStr">
         <is>
-          <t>2026/12/31</t>
+          <t>2026/12/30</t>
         </is>
       </c>
       <c r="B5006" t="inlineStr">
         <is>
-          <t>木</t>
+          <t>水</t>
         </is>
       </c>
       <c r="C5006" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D5006" t="n">
         <v>201</v>
@@ -90552,7 +90552,7 @@
         </is>
       </c>
       <c r="C5007" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="D5007" t="n">
         <v>201</v>
@@ -90570,7 +90570,7 @@
         </is>
       </c>
       <c r="C5008" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="D5008" t="n">
         <v>201</v>
@@ -90588,7 +90588,7 @@
         </is>
       </c>
       <c r="C5009" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="D5009" t="n">
         <v>201</v>
@@ -90606,7 +90606,7 @@
         </is>
       </c>
       <c r="C5010" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="D5010" t="n">
         <v>201</v>
@@ -90624,7 +90624,7 @@
         </is>
       </c>
       <c r="C5011" t="n">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="D5011" t="n">
         <v>201</v>
@@ -90633,16 +90633,16 @@
     <row r="5012">
       <c r="A5012" t="inlineStr">
         <is>
-          <t>2027/01/01</t>
+          <t>2026/12/31</t>
         </is>
       </c>
       <c r="B5012" t="inlineStr">
         <is>
-          <t>金</t>
+          <t>木</t>
         </is>
       </c>
       <c r="C5012" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D5012" t="n">
         <v>201</v>
@@ -90660,7 +90660,7 @@
         </is>
       </c>
       <c r="C5013" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D5013" t="n">
         <v>201</v>
@@ -90678,7 +90678,7 @@
         </is>
       </c>
       <c r="C5014" t="n">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="D5014" t="n">
         <v>201</v>
@@ -90696,7 +90696,7 @@
         </is>
       </c>
       <c r="C5015" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D5015" t="n">
         <v>201</v>
@@ -90714,7 +90714,7 @@
         </is>
       </c>
       <c r="C5016" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D5016" t="n">
         <v>201</v>
@@ -90723,16 +90723,16 @@
     <row r="5017">
       <c r="A5017" t="inlineStr">
         <is>
-          <t>2027/01/02</t>
+          <t>2027/01/01</t>
         </is>
       </c>
       <c r="B5017" t="inlineStr">
         <is>
-          <t>土</t>
+          <t>金</t>
         </is>
       </c>
       <c r="C5017" t="n">
-        <v>1</v>
+        <v>19</v>
       </c>
       <c r="D5017" t="n">
         <v>201</v>
@@ -90750,7 +90750,7 @@
         </is>
       </c>
       <c r="C5018" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D5018" t="n">
         <v>201</v>
@@ -90768,7 +90768,7 @@
         </is>
       </c>
       <c r="C5019" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D5019" t="n">
         <v>201</v>
@@ -90786,7 +90786,7 @@
         </is>
       </c>
       <c r="C5020" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="D5020" t="n">
         <v>201</v>
@@ -90804,7 +90804,7 @@
         </is>
       </c>
       <c r="C5021" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D5021" t="n">
         <v>201</v>
@@ -90822,7 +90822,7 @@
         </is>
       </c>
       <c r="C5022" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D5022" t="n">
         <v>201</v>
@@ -90840,7 +90840,7 @@
         </is>
       </c>
       <c r="C5023" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="D5023" t="n">
         <v>201</v>
@@ -90849,16 +90849,16 @@
     <row r="5024">
       <c r="A5024" t="inlineStr">
         <is>
-          <t>2027/01/03</t>
+          <t>2027/01/02</t>
         </is>
       </c>
       <c r="B5024" t="inlineStr">
         <is>
-          <t>日</t>
+          <t>土</t>
         </is>
       </c>
       <c r="C5024" t="n">
-        <v>1</v>
+        <v>22</v>
       </c>
       <c r="D5024" t="n">
         <v>201</v>
@@ -90876,7 +90876,7 @@
         </is>
       </c>
       <c r="C5025" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D5025" t="n">
         <v>201</v>
@@ -90894,7 +90894,7 @@
         </is>
       </c>
       <c r="C5026" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D5026" t="n">
         <v>201</v>
@@ -90912,7 +90912,7 @@
         </is>
       </c>
       <c r="C5027" t="n">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="D5027" t="n">
         <v>201</v>
@@ -90930,7 +90930,7 @@
         </is>
       </c>
       <c r="C5028" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D5028" t="n">
         <v>201</v>
@@ -90948,7 +90948,7 @@
         </is>
       </c>
       <c r="C5029" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D5029" t="n">
         <v>201</v>
@@ -90966,7 +90966,7 @@
         </is>
       </c>
       <c r="C5030" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="D5030" t="n">
         <v>201</v>
@@ -90975,16 +90975,16 @@
     <row r="5031">
       <c r="A5031" t="inlineStr">
         <is>
-          <t>2027/01/04</t>
+          <t>2027/01/03</t>
         </is>
       </c>
       <c r="B5031" t="inlineStr">
         <is>
-          <t>月</t>
+          <t>日</t>
         </is>
       </c>
       <c r="C5031" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D5031" t="n">
         <v>201</v>
@@ -91002,7 +91002,7 @@
         </is>
       </c>
       <c r="C5032" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D5032" t="n">
         <v>201</v>
@@ -91020,7 +91020,7 @@
         </is>
       </c>
       <c r="C5033" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D5033" t="n">
         <v>201</v>
@@ -91038,7 +91038,7 @@
         </is>
       </c>
       <c r="C5034" t="n">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="D5034" t="n">
         <v>201</v>
@@ -91056,7 +91056,7 @@
         </is>
       </c>
       <c r="C5035" t="n">
-        <v>22</v>
+        <v>13</v>
       </c>
       <c r="D5035" t="n">
         <v>201</v>
@@ -91065,16 +91065,16 @@
     <row r="5036">
       <c r="A5036" t="inlineStr">
         <is>
-          <t>2027/01/05</t>
+          <t>2027/01/04</t>
         </is>
       </c>
       <c r="B5036" t="inlineStr">
         <is>
-          <t>火</t>
+          <t>月</t>
         </is>
       </c>
       <c r="C5036" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D5036" t="n">
         <v>201</v>
@@ -91092,9 +91092,27 @@
         </is>
       </c>
       <c r="C5037" t="n">
+        <v>2</v>
+      </c>
+      <c r="D5037" t="n">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="5038">
+      <c r="A5038" t="inlineStr">
+        <is>
+          <t>2027/01/05</t>
+        </is>
+      </c>
+      <c r="B5038" t="inlineStr">
+        <is>
+          <t>火</t>
+        </is>
+      </c>
+      <c r="C5038" t="n">
         <v>7</v>
       </c>
-      <c r="D5037" t="n">
+      <c r="D5038" t="n">
         <v>201</v>
       </c>
     </row>

</xml_diff>

<commit_message>
daily auto push: 2026-09-25 08:45 UTC
</commit_message>
<xml_diff>
--- a/excel/apple2.xlsx
+++ b/excel/apple2.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D5070"/>
+  <dimension ref="A1:D5071"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -90939,16 +90939,16 @@
     <row r="5029">
       <c r="A5029" t="inlineStr">
         <is>
-          <t>2026/12/29</t>
+          <t>2026/09/25</t>
         </is>
       </c>
       <c r="B5029" t="inlineStr">
         <is>
-          <t>火</t>
+          <t>金</t>
         </is>
       </c>
       <c r="C5029" t="n">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="D5029" t="n">
         <v>201</v>
@@ -90966,7 +90966,7 @@
         </is>
       </c>
       <c r="C5030" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D5030" t="n">
         <v>201</v>
@@ -90984,7 +90984,7 @@
         </is>
       </c>
       <c r="C5031" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D5031" t="n">
         <v>201</v>
@@ -91002,7 +91002,7 @@
         </is>
       </c>
       <c r="C5032" t="n">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="D5032" t="n">
         <v>201</v>
@@ -91011,16 +91011,16 @@
     <row r="5033">
       <c r="A5033" t="inlineStr">
         <is>
-          <t>2026/12/30</t>
+          <t>2026/12/29</t>
         </is>
       </c>
       <c r="B5033" t="inlineStr">
         <is>
-          <t>水</t>
+          <t>火</t>
         </is>
       </c>
       <c r="C5033" t="n">
-        <v>2</v>
+        <v>23</v>
       </c>
       <c r="D5033" t="n">
         <v>201</v>
@@ -91038,7 +91038,7 @@
         </is>
       </c>
       <c r="C5034" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D5034" t="n">
         <v>201</v>
@@ -91056,7 +91056,7 @@
         </is>
       </c>
       <c r="C5035" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D5035" t="n">
         <v>201</v>
@@ -91074,7 +91074,7 @@
         </is>
       </c>
       <c r="C5036" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="D5036" t="n">
         <v>201</v>
@@ -91092,7 +91092,7 @@
         </is>
       </c>
       <c r="C5037" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D5037" t="n">
         <v>201</v>
@@ -91110,7 +91110,7 @@
         </is>
       </c>
       <c r="C5038" t="n">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="D5038" t="n">
         <v>201</v>
@@ -91119,16 +91119,16 @@
     <row r="5039">
       <c r="A5039" t="inlineStr">
         <is>
-          <t>2026/12/31</t>
+          <t>2026/12/30</t>
         </is>
       </c>
       <c r="B5039" t="inlineStr">
         <is>
-          <t>木</t>
+          <t>水</t>
         </is>
       </c>
       <c r="C5039" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D5039" t="n">
         <v>201</v>
@@ -91146,7 +91146,7 @@
         </is>
       </c>
       <c r="C5040" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="D5040" t="n">
         <v>201</v>
@@ -91164,7 +91164,7 @@
         </is>
       </c>
       <c r="C5041" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="D5041" t="n">
         <v>201</v>
@@ -91182,7 +91182,7 @@
         </is>
       </c>
       <c r="C5042" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="D5042" t="n">
         <v>201</v>
@@ -91200,7 +91200,7 @@
         </is>
       </c>
       <c r="C5043" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="D5043" t="n">
         <v>201</v>
@@ -91218,7 +91218,7 @@
         </is>
       </c>
       <c r="C5044" t="n">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="D5044" t="n">
         <v>201</v>
@@ -91227,16 +91227,16 @@
     <row r="5045">
       <c r="A5045" t="inlineStr">
         <is>
-          <t>2027/01/01</t>
+          <t>2026/12/31</t>
         </is>
       </c>
       <c r="B5045" t="inlineStr">
         <is>
-          <t>金</t>
+          <t>木</t>
         </is>
       </c>
       <c r="C5045" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D5045" t="n">
         <v>201</v>
@@ -91254,7 +91254,7 @@
         </is>
       </c>
       <c r="C5046" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D5046" t="n">
         <v>201</v>
@@ -91272,7 +91272,7 @@
         </is>
       </c>
       <c r="C5047" t="n">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="D5047" t="n">
         <v>201</v>
@@ -91290,7 +91290,7 @@
         </is>
       </c>
       <c r="C5048" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D5048" t="n">
         <v>201</v>
@@ -91308,7 +91308,7 @@
         </is>
       </c>
       <c r="C5049" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D5049" t="n">
         <v>201</v>
@@ -91317,16 +91317,16 @@
     <row r="5050">
       <c r="A5050" t="inlineStr">
         <is>
-          <t>2027/01/02</t>
+          <t>2027/01/01</t>
         </is>
       </c>
       <c r="B5050" t="inlineStr">
         <is>
-          <t>土</t>
+          <t>金</t>
         </is>
       </c>
       <c r="C5050" t="n">
-        <v>1</v>
+        <v>19</v>
       </c>
       <c r="D5050" t="n">
         <v>201</v>
@@ -91344,7 +91344,7 @@
         </is>
       </c>
       <c r="C5051" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D5051" t="n">
         <v>201</v>
@@ -91362,7 +91362,7 @@
         </is>
       </c>
       <c r="C5052" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D5052" t="n">
         <v>201</v>
@@ -91380,7 +91380,7 @@
         </is>
       </c>
       <c r="C5053" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="D5053" t="n">
         <v>201</v>
@@ -91398,7 +91398,7 @@
         </is>
       </c>
       <c r="C5054" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D5054" t="n">
         <v>201</v>
@@ -91416,7 +91416,7 @@
         </is>
       </c>
       <c r="C5055" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D5055" t="n">
         <v>201</v>
@@ -91434,7 +91434,7 @@
         </is>
       </c>
       <c r="C5056" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="D5056" t="n">
         <v>201</v>
@@ -91443,16 +91443,16 @@
     <row r="5057">
       <c r="A5057" t="inlineStr">
         <is>
-          <t>2027/01/03</t>
+          <t>2027/01/02</t>
         </is>
       </c>
       <c r="B5057" t="inlineStr">
         <is>
-          <t>日</t>
+          <t>土</t>
         </is>
       </c>
       <c r="C5057" t="n">
-        <v>1</v>
+        <v>22</v>
       </c>
       <c r="D5057" t="n">
         <v>201</v>
@@ -91470,7 +91470,7 @@
         </is>
       </c>
       <c r="C5058" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D5058" t="n">
         <v>201</v>
@@ -91488,7 +91488,7 @@
         </is>
       </c>
       <c r="C5059" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D5059" t="n">
         <v>201</v>
@@ -91506,7 +91506,7 @@
         </is>
       </c>
       <c r="C5060" t="n">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="D5060" t="n">
         <v>201</v>
@@ -91524,7 +91524,7 @@
         </is>
       </c>
       <c r="C5061" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D5061" t="n">
         <v>201</v>
@@ -91542,7 +91542,7 @@
         </is>
       </c>
       <c r="C5062" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D5062" t="n">
         <v>201</v>
@@ -91560,7 +91560,7 @@
         </is>
       </c>
       <c r="C5063" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="D5063" t="n">
         <v>201</v>
@@ -91569,16 +91569,16 @@
     <row r="5064">
       <c r="A5064" t="inlineStr">
         <is>
-          <t>2027/01/04</t>
+          <t>2027/01/03</t>
         </is>
       </c>
       <c r="B5064" t="inlineStr">
         <is>
-          <t>月</t>
+          <t>日</t>
         </is>
       </c>
       <c r="C5064" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D5064" t="n">
         <v>201</v>
@@ -91596,7 +91596,7 @@
         </is>
       </c>
       <c r="C5065" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D5065" t="n">
         <v>201</v>
@@ -91614,7 +91614,7 @@
         </is>
       </c>
       <c r="C5066" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D5066" t="n">
         <v>201</v>
@@ -91632,7 +91632,7 @@
         </is>
       </c>
       <c r="C5067" t="n">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="D5067" t="n">
         <v>201</v>
@@ -91650,7 +91650,7 @@
         </is>
       </c>
       <c r="C5068" t="n">
-        <v>22</v>
+        <v>13</v>
       </c>
       <c r="D5068" t="n">
         <v>201</v>
@@ -91659,16 +91659,16 @@
     <row r="5069">
       <c r="A5069" t="inlineStr">
         <is>
-          <t>2027/01/05</t>
+          <t>2027/01/04</t>
         </is>
       </c>
       <c r="B5069" t="inlineStr">
         <is>
-          <t>火</t>
+          <t>月</t>
         </is>
       </c>
       <c r="C5069" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D5069" t="n">
         <v>201</v>
@@ -91686,9 +91686,27 @@
         </is>
       </c>
       <c r="C5070" t="n">
+        <v>2</v>
+      </c>
+      <c r="D5070" t="n">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="5071">
+      <c r="A5071" t="inlineStr">
+        <is>
+          <t>2027/01/05</t>
+        </is>
+      </c>
+      <c r="B5071" t="inlineStr">
+        <is>
+          <t>火</t>
+        </is>
+      </c>
+      <c r="C5071" t="n">
         <v>7</v>
       </c>
-      <c r="D5070" t="n">
+      <c r="D5071" t="n">
         <v>201</v>
       </c>
     </row>

</xml_diff>

<commit_message>
daily auto push: 2026-09-30 15:52 UTC
</commit_message>
<xml_diff>
--- a/excel/apple2.xlsx
+++ b/excel/apple2.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D5109"/>
+  <dimension ref="A1:D5110"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -91641,16 +91641,16 @@
     <row r="5068">
       <c r="A5068" t="inlineStr">
         <is>
-          <t>2026/12/29</t>
+          <t>2026/09/30</t>
         </is>
       </c>
       <c r="B5068" t="inlineStr">
         <is>
-          <t>火</t>
+          <t>水</t>
         </is>
       </c>
       <c r="C5068" t="n">
-        <v>13</v>
+        <v>23</v>
       </c>
       <c r="D5068" t="n">
         <v>201</v>
@@ -91668,7 +91668,7 @@
         </is>
       </c>
       <c r="C5069" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D5069" t="n">
         <v>201</v>
@@ -91686,7 +91686,7 @@
         </is>
       </c>
       <c r="C5070" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D5070" t="n">
         <v>201</v>
@@ -91704,7 +91704,7 @@
         </is>
       </c>
       <c r="C5071" t="n">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="D5071" t="n">
         <v>201</v>
@@ -91713,16 +91713,16 @@
     <row r="5072">
       <c r="A5072" t="inlineStr">
         <is>
-          <t>2026/12/30</t>
+          <t>2026/12/29</t>
         </is>
       </c>
       <c r="B5072" t="inlineStr">
         <is>
-          <t>水</t>
+          <t>火</t>
         </is>
       </c>
       <c r="C5072" t="n">
-        <v>2</v>
+        <v>23</v>
       </c>
       <c r="D5072" t="n">
         <v>201</v>
@@ -91740,7 +91740,7 @@
         </is>
       </c>
       <c r="C5073" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D5073" t="n">
         <v>201</v>
@@ -91758,7 +91758,7 @@
         </is>
       </c>
       <c r="C5074" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D5074" t="n">
         <v>201</v>
@@ -91776,7 +91776,7 @@
         </is>
       </c>
       <c r="C5075" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="D5075" t="n">
         <v>201</v>
@@ -91794,7 +91794,7 @@
         </is>
       </c>
       <c r="C5076" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D5076" t="n">
         <v>201</v>
@@ -91812,7 +91812,7 @@
         </is>
       </c>
       <c r="C5077" t="n">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="D5077" t="n">
         <v>201</v>
@@ -91821,16 +91821,16 @@
     <row r="5078">
       <c r="A5078" t="inlineStr">
         <is>
-          <t>2026/12/31</t>
+          <t>2026/12/30</t>
         </is>
       </c>
       <c r="B5078" t="inlineStr">
         <is>
-          <t>木</t>
+          <t>水</t>
         </is>
       </c>
       <c r="C5078" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D5078" t="n">
         <v>201</v>
@@ -91848,7 +91848,7 @@
         </is>
       </c>
       <c r="C5079" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="D5079" t="n">
         <v>201</v>
@@ -91866,7 +91866,7 @@
         </is>
       </c>
       <c r="C5080" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="D5080" t="n">
         <v>201</v>
@@ -91884,7 +91884,7 @@
         </is>
       </c>
       <c r="C5081" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="D5081" t="n">
         <v>201</v>
@@ -91902,7 +91902,7 @@
         </is>
       </c>
       <c r="C5082" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="D5082" t="n">
         <v>201</v>
@@ -91920,7 +91920,7 @@
         </is>
       </c>
       <c r="C5083" t="n">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="D5083" t="n">
         <v>201</v>
@@ -91929,16 +91929,16 @@
     <row r="5084">
       <c r="A5084" t="inlineStr">
         <is>
-          <t>2027/01/01</t>
+          <t>2026/12/31</t>
         </is>
       </c>
       <c r="B5084" t="inlineStr">
         <is>
-          <t>金</t>
+          <t>木</t>
         </is>
       </c>
       <c r="C5084" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D5084" t="n">
         <v>201</v>
@@ -91956,7 +91956,7 @@
         </is>
       </c>
       <c r="C5085" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D5085" t="n">
         <v>201</v>
@@ -91974,7 +91974,7 @@
         </is>
       </c>
       <c r="C5086" t="n">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="D5086" t="n">
         <v>201</v>
@@ -91992,7 +91992,7 @@
         </is>
       </c>
       <c r="C5087" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D5087" t="n">
         <v>201</v>
@@ -92010,7 +92010,7 @@
         </is>
       </c>
       <c r="C5088" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D5088" t="n">
         <v>201</v>
@@ -92019,16 +92019,16 @@
     <row r="5089">
       <c r="A5089" t="inlineStr">
         <is>
-          <t>2027/01/02</t>
+          <t>2027/01/01</t>
         </is>
       </c>
       <c r="B5089" t="inlineStr">
         <is>
-          <t>土</t>
+          <t>金</t>
         </is>
       </c>
       <c r="C5089" t="n">
-        <v>1</v>
+        <v>19</v>
       </c>
       <c r="D5089" t="n">
         <v>201</v>
@@ -92046,7 +92046,7 @@
         </is>
       </c>
       <c r="C5090" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D5090" t="n">
         <v>201</v>
@@ -92064,7 +92064,7 @@
         </is>
       </c>
       <c r="C5091" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D5091" t="n">
         <v>201</v>
@@ -92082,7 +92082,7 @@
         </is>
       </c>
       <c r="C5092" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="D5092" t="n">
         <v>201</v>
@@ -92100,7 +92100,7 @@
         </is>
       </c>
       <c r="C5093" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D5093" t="n">
         <v>201</v>
@@ -92118,7 +92118,7 @@
         </is>
       </c>
       <c r="C5094" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D5094" t="n">
         <v>201</v>
@@ -92136,7 +92136,7 @@
         </is>
       </c>
       <c r="C5095" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="D5095" t="n">
         <v>201</v>
@@ -92145,16 +92145,16 @@
     <row r="5096">
       <c r="A5096" t="inlineStr">
         <is>
-          <t>2027/01/03</t>
+          <t>2027/01/02</t>
         </is>
       </c>
       <c r="B5096" t="inlineStr">
         <is>
-          <t>日</t>
+          <t>土</t>
         </is>
       </c>
       <c r="C5096" t="n">
-        <v>1</v>
+        <v>22</v>
       </c>
       <c r="D5096" t="n">
         <v>201</v>
@@ -92172,7 +92172,7 @@
         </is>
       </c>
       <c r="C5097" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D5097" t="n">
         <v>201</v>
@@ -92190,7 +92190,7 @@
         </is>
       </c>
       <c r="C5098" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D5098" t="n">
         <v>201</v>
@@ -92208,7 +92208,7 @@
         </is>
       </c>
       <c r="C5099" t="n">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="D5099" t="n">
         <v>201</v>
@@ -92226,7 +92226,7 @@
         </is>
       </c>
       <c r="C5100" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D5100" t="n">
         <v>201</v>
@@ -92244,7 +92244,7 @@
         </is>
       </c>
       <c r="C5101" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D5101" t="n">
         <v>201</v>
@@ -92262,7 +92262,7 @@
         </is>
       </c>
       <c r="C5102" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="D5102" t="n">
         <v>201</v>
@@ -92271,16 +92271,16 @@
     <row r="5103">
       <c r="A5103" t="inlineStr">
         <is>
-          <t>2027/01/04</t>
+          <t>2027/01/03</t>
         </is>
       </c>
       <c r="B5103" t="inlineStr">
         <is>
-          <t>月</t>
+          <t>日</t>
         </is>
       </c>
       <c r="C5103" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D5103" t="n">
         <v>201</v>
@@ -92298,7 +92298,7 @@
         </is>
       </c>
       <c r="C5104" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D5104" t="n">
         <v>201</v>
@@ -92316,7 +92316,7 @@
         </is>
       </c>
       <c r="C5105" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D5105" t="n">
         <v>201</v>
@@ -92334,7 +92334,7 @@
         </is>
       </c>
       <c r="C5106" t="n">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="D5106" t="n">
         <v>201</v>
@@ -92352,7 +92352,7 @@
         </is>
       </c>
       <c r="C5107" t="n">
-        <v>22</v>
+        <v>13</v>
       </c>
       <c r="D5107" t="n">
         <v>201</v>
@@ -92361,16 +92361,16 @@
     <row r="5108">
       <c r="A5108" t="inlineStr">
         <is>
-          <t>2027/01/05</t>
+          <t>2027/01/04</t>
         </is>
       </c>
       <c r="B5108" t="inlineStr">
         <is>
-          <t>火</t>
+          <t>月</t>
         </is>
       </c>
       <c r="C5108" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D5108" t="n">
         <v>201</v>
@@ -92388,9 +92388,27 @@
         </is>
       </c>
       <c r="C5109" t="n">
+        <v>2</v>
+      </c>
+      <c r="D5109" t="n">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="5110">
+      <c r="A5110" t="inlineStr">
+        <is>
+          <t>2027/01/05</t>
+        </is>
+      </c>
+      <c r="B5110" t="inlineStr">
+        <is>
+          <t>火</t>
+        </is>
+      </c>
+      <c r="C5110" t="n">
         <v>7</v>
       </c>
-      <c r="D5109" t="n">
+      <c r="D5110" t="n">
         <v>201</v>
       </c>
     </row>

</xml_diff>

<commit_message>
daily auto push: 2026-10-01 14:25 UTC
</commit_message>
<xml_diff>
--- a/excel/apple2.xlsx
+++ b/excel/apple2.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D5116"/>
+  <dimension ref="A1:D5117"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -91767,16 +91767,16 @@
     <row r="5075">
       <c r="A5075" t="inlineStr">
         <is>
-          <t>2026/12/29</t>
+          <t>2026/10/01</t>
         </is>
       </c>
       <c r="B5075" t="inlineStr">
         <is>
-          <t>火</t>
+          <t>木</t>
         </is>
       </c>
       <c r="C5075" t="n">
-        <v>13</v>
+        <v>23</v>
       </c>
       <c r="D5075" t="n">
         <v>201</v>
@@ -91794,7 +91794,7 @@
         </is>
       </c>
       <c r="C5076" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D5076" t="n">
         <v>201</v>
@@ -91812,7 +91812,7 @@
         </is>
       </c>
       <c r="C5077" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D5077" t="n">
         <v>201</v>
@@ -91830,7 +91830,7 @@
         </is>
       </c>
       <c r="C5078" t="n">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="D5078" t="n">
         <v>201</v>
@@ -91839,16 +91839,16 @@
     <row r="5079">
       <c r="A5079" t="inlineStr">
         <is>
-          <t>2026/12/30</t>
+          <t>2026/12/29</t>
         </is>
       </c>
       <c r="B5079" t="inlineStr">
         <is>
-          <t>水</t>
+          <t>火</t>
         </is>
       </c>
       <c r="C5079" t="n">
-        <v>2</v>
+        <v>23</v>
       </c>
       <c r="D5079" t="n">
         <v>201</v>
@@ -91866,7 +91866,7 @@
         </is>
       </c>
       <c r="C5080" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D5080" t="n">
         <v>201</v>
@@ -91884,7 +91884,7 @@
         </is>
       </c>
       <c r="C5081" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D5081" t="n">
         <v>201</v>
@@ -91902,7 +91902,7 @@
         </is>
       </c>
       <c r="C5082" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="D5082" t="n">
         <v>201</v>
@@ -91920,7 +91920,7 @@
         </is>
       </c>
       <c r="C5083" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D5083" t="n">
         <v>201</v>
@@ -91938,7 +91938,7 @@
         </is>
       </c>
       <c r="C5084" t="n">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="D5084" t="n">
         <v>201</v>
@@ -91947,16 +91947,16 @@
     <row r="5085">
       <c r="A5085" t="inlineStr">
         <is>
-          <t>2026/12/31</t>
+          <t>2026/12/30</t>
         </is>
       </c>
       <c r="B5085" t="inlineStr">
         <is>
-          <t>木</t>
+          <t>水</t>
         </is>
       </c>
       <c r="C5085" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D5085" t="n">
         <v>201</v>
@@ -91974,7 +91974,7 @@
         </is>
       </c>
       <c r="C5086" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="D5086" t="n">
         <v>201</v>
@@ -91992,7 +91992,7 @@
         </is>
       </c>
       <c r="C5087" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="D5087" t="n">
         <v>201</v>
@@ -92010,7 +92010,7 @@
         </is>
       </c>
       <c r="C5088" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="D5088" t="n">
         <v>201</v>
@@ -92028,7 +92028,7 @@
         </is>
       </c>
       <c r="C5089" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="D5089" t="n">
         <v>201</v>
@@ -92046,7 +92046,7 @@
         </is>
       </c>
       <c r="C5090" t="n">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="D5090" t="n">
         <v>201</v>
@@ -92055,16 +92055,16 @@
     <row r="5091">
       <c r="A5091" t="inlineStr">
         <is>
-          <t>2027/01/01</t>
+          <t>2026/12/31</t>
         </is>
       </c>
       <c r="B5091" t="inlineStr">
         <is>
-          <t>金</t>
+          <t>木</t>
         </is>
       </c>
       <c r="C5091" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D5091" t="n">
         <v>201</v>
@@ -92082,7 +92082,7 @@
         </is>
       </c>
       <c r="C5092" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D5092" t="n">
         <v>201</v>
@@ -92100,7 +92100,7 @@
         </is>
       </c>
       <c r="C5093" t="n">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="D5093" t="n">
         <v>201</v>
@@ -92118,7 +92118,7 @@
         </is>
       </c>
       <c r="C5094" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D5094" t="n">
         <v>201</v>
@@ -92136,7 +92136,7 @@
         </is>
       </c>
       <c r="C5095" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D5095" t="n">
         <v>201</v>
@@ -92145,16 +92145,16 @@
     <row r="5096">
       <c r="A5096" t="inlineStr">
         <is>
-          <t>2027/01/02</t>
+          <t>2027/01/01</t>
         </is>
       </c>
       <c r="B5096" t="inlineStr">
         <is>
-          <t>土</t>
+          <t>金</t>
         </is>
       </c>
       <c r="C5096" t="n">
-        <v>1</v>
+        <v>19</v>
       </c>
       <c r="D5096" t="n">
         <v>201</v>
@@ -92172,7 +92172,7 @@
         </is>
       </c>
       <c r="C5097" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D5097" t="n">
         <v>201</v>
@@ -92190,7 +92190,7 @@
         </is>
       </c>
       <c r="C5098" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D5098" t="n">
         <v>201</v>
@@ -92208,7 +92208,7 @@
         </is>
       </c>
       <c r="C5099" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="D5099" t="n">
         <v>201</v>
@@ -92226,7 +92226,7 @@
         </is>
       </c>
       <c r="C5100" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D5100" t="n">
         <v>201</v>
@@ -92244,7 +92244,7 @@
         </is>
       </c>
       <c r="C5101" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D5101" t="n">
         <v>201</v>
@@ -92262,7 +92262,7 @@
         </is>
       </c>
       <c r="C5102" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="D5102" t="n">
         <v>201</v>
@@ -92271,16 +92271,16 @@
     <row r="5103">
       <c r="A5103" t="inlineStr">
         <is>
-          <t>2027/01/03</t>
+          <t>2027/01/02</t>
         </is>
       </c>
       <c r="B5103" t="inlineStr">
         <is>
-          <t>日</t>
+          <t>土</t>
         </is>
       </c>
       <c r="C5103" t="n">
-        <v>1</v>
+        <v>22</v>
       </c>
       <c r="D5103" t="n">
         <v>201</v>
@@ -92298,7 +92298,7 @@
         </is>
       </c>
       <c r="C5104" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D5104" t="n">
         <v>201</v>
@@ -92316,7 +92316,7 @@
         </is>
       </c>
       <c r="C5105" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D5105" t="n">
         <v>201</v>
@@ -92334,7 +92334,7 @@
         </is>
       </c>
       <c r="C5106" t="n">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="D5106" t="n">
         <v>201</v>
@@ -92352,7 +92352,7 @@
         </is>
       </c>
       <c r="C5107" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D5107" t="n">
         <v>201</v>
@@ -92370,7 +92370,7 @@
         </is>
       </c>
       <c r="C5108" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D5108" t="n">
         <v>201</v>
@@ -92388,7 +92388,7 @@
         </is>
       </c>
       <c r="C5109" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="D5109" t="n">
         <v>201</v>
@@ -92397,16 +92397,16 @@
     <row r="5110">
       <c r="A5110" t="inlineStr">
         <is>
-          <t>2027/01/04</t>
+          <t>2027/01/03</t>
         </is>
       </c>
       <c r="B5110" t="inlineStr">
         <is>
-          <t>月</t>
+          <t>日</t>
         </is>
       </c>
       <c r="C5110" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D5110" t="n">
         <v>201</v>
@@ -92424,7 +92424,7 @@
         </is>
       </c>
       <c r="C5111" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D5111" t="n">
         <v>201</v>
@@ -92442,7 +92442,7 @@
         </is>
       </c>
       <c r="C5112" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D5112" t="n">
         <v>201</v>
@@ -92460,7 +92460,7 @@
         </is>
       </c>
       <c r="C5113" t="n">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="D5113" t="n">
         <v>201</v>
@@ -92478,7 +92478,7 @@
         </is>
       </c>
       <c r="C5114" t="n">
-        <v>22</v>
+        <v>13</v>
       </c>
       <c r="D5114" t="n">
         <v>201</v>
@@ -92487,16 +92487,16 @@
     <row r="5115">
       <c r="A5115" t="inlineStr">
         <is>
-          <t>2027/01/05</t>
+          <t>2027/01/04</t>
         </is>
       </c>
       <c r="B5115" t="inlineStr">
         <is>
-          <t>火</t>
+          <t>月</t>
         </is>
       </c>
       <c r="C5115" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D5115" t="n">
         <v>201</v>
@@ -92514,9 +92514,27 @@
         </is>
       </c>
       <c r="C5116" t="n">
+        <v>2</v>
+      </c>
+      <c r="D5116" t="n">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="5117">
+      <c r="A5117" t="inlineStr">
+        <is>
+          <t>2027/01/05</t>
+        </is>
+      </c>
+      <c r="B5117" t="inlineStr">
+        <is>
+          <t>火</t>
+        </is>
+      </c>
+      <c r="C5117" t="n">
         <v>7</v>
       </c>
-      <c r="D5116" t="n">
+      <c r="D5117" t="n">
         <v>201</v>
       </c>
     </row>

</xml_diff>

<commit_message>
daily auto push: 2026-10-01 18:51 UTC
</commit_message>
<xml_diff>
--- a/excel/apple2.xlsx
+++ b/excel/apple2.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D5117"/>
+  <dimension ref="A1:D5118"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -91785,16 +91785,16 @@
     <row r="5076">
       <c r="A5076" t="inlineStr">
         <is>
-          <t>2026/12/29</t>
+          <t>2026/10/02</t>
         </is>
       </c>
       <c r="B5076" t="inlineStr">
         <is>
-          <t>火</t>
+          <t>金</t>
         </is>
       </c>
       <c r="C5076" t="n">
-        <v>13</v>
+        <v>2</v>
       </c>
       <c r="D5076" t="n">
         <v>201</v>
@@ -91812,7 +91812,7 @@
         </is>
       </c>
       <c r="C5077" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D5077" t="n">
         <v>201</v>
@@ -91830,7 +91830,7 @@
         </is>
       </c>
       <c r="C5078" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D5078" t="n">
         <v>201</v>
@@ -91848,7 +91848,7 @@
         </is>
       </c>
       <c r="C5079" t="n">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="D5079" t="n">
         <v>201</v>
@@ -91857,16 +91857,16 @@
     <row r="5080">
       <c r="A5080" t="inlineStr">
         <is>
-          <t>2026/12/30</t>
+          <t>2026/12/29</t>
         </is>
       </c>
       <c r="B5080" t="inlineStr">
         <is>
-          <t>水</t>
+          <t>火</t>
         </is>
       </c>
       <c r="C5080" t="n">
-        <v>2</v>
+        <v>23</v>
       </c>
       <c r="D5080" t="n">
         <v>201</v>
@@ -91884,7 +91884,7 @@
         </is>
       </c>
       <c r="C5081" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D5081" t="n">
         <v>201</v>
@@ -91902,7 +91902,7 @@
         </is>
       </c>
       <c r="C5082" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D5082" t="n">
         <v>201</v>
@@ -91920,7 +91920,7 @@
         </is>
       </c>
       <c r="C5083" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="D5083" t="n">
         <v>201</v>
@@ -91938,7 +91938,7 @@
         </is>
       </c>
       <c r="C5084" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D5084" t="n">
         <v>201</v>
@@ -91956,7 +91956,7 @@
         </is>
       </c>
       <c r="C5085" t="n">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="D5085" t="n">
         <v>201</v>
@@ -91965,16 +91965,16 @@
     <row r="5086">
       <c r="A5086" t="inlineStr">
         <is>
-          <t>2026/12/31</t>
+          <t>2026/12/30</t>
         </is>
       </c>
       <c r="B5086" t="inlineStr">
         <is>
-          <t>木</t>
+          <t>水</t>
         </is>
       </c>
       <c r="C5086" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D5086" t="n">
         <v>201</v>
@@ -91992,7 +91992,7 @@
         </is>
       </c>
       <c r="C5087" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="D5087" t="n">
         <v>201</v>
@@ -92010,7 +92010,7 @@
         </is>
       </c>
       <c r="C5088" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="D5088" t="n">
         <v>201</v>
@@ -92028,7 +92028,7 @@
         </is>
       </c>
       <c r="C5089" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="D5089" t="n">
         <v>201</v>
@@ -92046,7 +92046,7 @@
         </is>
       </c>
       <c r="C5090" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="D5090" t="n">
         <v>201</v>
@@ -92064,7 +92064,7 @@
         </is>
       </c>
       <c r="C5091" t="n">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="D5091" t="n">
         <v>201</v>
@@ -92073,16 +92073,16 @@
     <row r="5092">
       <c r="A5092" t="inlineStr">
         <is>
-          <t>2027/01/01</t>
+          <t>2026/12/31</t>
         </is>
       </c>
       <c r="B5092" t="inlineStr">
         <is>
-          <t>金</t>
+          <t>木</t>
         </is>
       </c>
       <c r="C5092" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D5092" t="n">
         <v>201</v>
@@ -92100,7 +92100,7 @@
         </is>
       </c>
       <c r="C5093" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D5093" t="n">
         <v>201</v>
@@ -92118,7 +92118,7 @@
         </is>
       </c>
       <c r="C5094" t="n">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="D5094" t="n">
         <v>201</v>
@@ -92136,7 +92136,7 @@
         </is>
       </c>
       <c r="C5095" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D5095" t="n">
         <v>201</v>
@@ -92154,7 +92154,7 @@
         </is>
       </c>
       <c r="C5096" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D5096" t="n">
         <v>201</v>
@@ -92163,16 +92163,16 @@
     <row r="5097">
       <c r="A5097" t="inlineStr">
         <is>
-          <t>2027/01/02</t>
+          <t>2027/01/01</t>
         </is>
       </c>
       <c r="B5097" t="inlineStr">
         <is>
-          <t>土</t>
+          <t>金</t>
         </is>
       </c>
       <c r="C5097" t="n">
-        <v>1</v>
+        <v>19</v>
       </c>
       <c r="D5097" t="n">
         <v>201</v>
@@ -92190,7 +92190,7 @@
         </is>
       </c>
       <c r="C5098" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D5098" t="n">
         <v>201</v>
@@ -92208,7 +92208,7 @@
         </is>
       </c>
       <c r="C5099" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D5099" t="n">
         <v>201</v>
@@ -92226,7 +92226,7 @@
         </is>
       </c>
       <c r="C5100" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="D5100" t="n">
         <v>201</v>
@@ -92244,7 +92244,7 @@
         </is>
       </c>
       <c r="C5101" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D5101" t="n">
         <v>201</v>
@@ -92262,7 +92262,7 @@
         </is>
       </c>
       <c r="C5102" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D5102" t="n">
         <v>201</v>
@@ -92280,7 +92280,7 @@
         </is>
       </c>
       <c r="C5103" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="D5103" t="n">
         <v>201</v>
@@ -92289,16 +92289,16 @@
     <row r="5104">
       <c r="A5104" t="inlineStr">
         <is>
-          <t>2027/01/03</t>
+          <t>2027/01/02</t>
         </is>
       </c>
       <c r="B5104" t="inlineStr">
         <is>
-          <t>日</t>
+          <t>土</t>
         </is>
       </c>
       <c r="C5104" t="n">
-        <v>1</v>
+        <v>22</v>
       </c>
       <c r="D5104" t="n">
         <v>201</v>
@@ -92316,7 +92316,7 @@
         </is>
       </c>
       <c r="C5105" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D5105" t="n">
         <v>201</v>
@@ -92334,7 +92334,7 @@
         </is>
       </c>
       <c r="C5106" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D5106" t="n">
         <v>201</v>
@@ -92352,7 +92352,7 @@
         </is>
       </c>
       <c r="C5107" t="n">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="D5107" t="n">
         <v>201</v>
@@ -92370,7 +92370,7 @@
         </is>
       </c>
       <c r="C5108" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D5108" t="n">
         <v>201</v>
@@ -92388,7 +92388,7 @@
         </is>
       </c>
       <c r="C5109" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D5109" t="n">
         <v>201</v>
@@ -92406,7 +92406,7 @@
         </is>
       </c>
       <c r="C5110" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="D5110" t="n">
         <v>201</v>
@@ -92415,16 +92415,16 @@
     <row r="5111">
       <c r="A5111" t="inlineStr">
         <is>
-          <t>2027/01/04</t>
+          <t>2027/01/03</t>
         </is>
       </c>
       <c r="B5111" t="inlineStr">
         <is>
-          <t>月</t>
+          <t>日</t>
         </is>
       </c>
       <c r="C5111" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D5111" t="n">
         <v>201</v>
@@ -92442,7 +92442,7 @@
         </is>
       </c>
       <c r="C5112" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D5112" t="n">
         <v>201</v>
@@ -92460,7 +92460,7 @@
         </is>
       </c>
       <c r="C5113" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D5113" t="n">
         <v>201</v>
@@ -92478,7 +92478,7 @@
         </is>
       </c>
       <c r="C5114" t="n">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="D5114" t="n">
         <v>201</v>
@@ -92496,7 +92496,7 @@
         </is>
       </c>
       <c r="C5115" t="n">
-        <v>22</v>
+        <v>13</v>
       </c>
       <c r="D5115" t="n">
         <v>201</v>
@@ -92505,16 +92505,16 @@
     <row r="5116">
       <c r="A5116" t="inlineStr">
         <is>
-          <t>2027/01/05</t>
+          <t>2027/01/04</t>
         </is>
       </c>
       <c r="B5116" t="inlineStr">
         <is>
-          <t>火</t>
+          <t>月</t>
         </is>
       </c>
       <c r="C5116" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D5116" t="n">
         <v>201</v>
@@ -92532,9 +92532,27 @@
         </is>
       </c>
       <c r="C5117" t="n">
+        <v>2</v>
+      </c>
+      <c r="D5117" t="n">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="5118">
+      <c r="A5118" t="inlineStr">
+        <is>
+          <t>2027/01/05</t>
+        </is>
+      </c>
+      <c r="B5118" t="inlineStr">
+        <is>
+          <t>火</t>
+        </is>
+      </c>
+      <c r="C5118" t="n">
         <v>7</v>
       </c>
-      <c r="D5117" t="n">
+      <c r="D5118" t="n">
         <v>201</v>
       </c>
     </row>

</xml_diff>

<commit_message>
daily auto push: 2026-10-03 09:05 UTC
</commit_message>
<xml_diff>
--- a/excel/apple2.xlsx
+++ b/excel/apple2.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D5129"/>
+  <dimension ref="A1:D5130"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -92001,16 +92001,16 @@
     <row r="5088">
       <c r="A5088" t="inlineStr">
         <is>
-          <t>2026/12/29</t>
+          <t>2026/10/03</t>
         </is>
       </c>
       <c r="B5088" t="inlineStr">
         <is>
-          <t>火</t>
+          <t>土</t>
         </is>
       </c>
       <c r="C5088" t="n">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="D5088" t="n">
         <v>201</v>
@@ -92028,7 +92028,7 @@
         </is>
       </c>
       <c r="C5089" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D5089" t="n">
         <v>201</v>
@@ -92046,7 +92046,7 @@
         </is>
       </c>
       <c r="C5090" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D5090" t="n">
         <v>201</v>
@@ -92064,7 +92064,7 @@
         </is>
       </c>
       <c r="C5091" t="n">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="D5091" t="n">
         <v>201</v>
@@ -92073,16 +92073,16 @@
     <row r="5092">
       <c r="A5092" t="inlineStr">
         <is>
-          <t>2026/12/30</t>
+          <t>2026/12/29</t>
         </is>
       </c>
       <c r="B5092" t="inlineStr">
         <is>
-          <t>水</t>
+          <t>火</t>
         </is>
       </c>
       <c r="C5092" t="n">
-        <v>2</v>
+        <v>23</v>
       </c>
       <c r="D5092" t="n">
         <v>201</v>
@@ -92100,7 +92100,7 @@
         </is>
       </c>
       <c r="C5093" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D5093" t="n">
         <v>201</v>
@@ -92118,7 +92118,7 @@
         </is>
       </c>
       <c r="C5094" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D5094" t="n">
         <v>201</v>
@@ -92136,7 +92136,7 @@
         </is>
       </c>
       <c r="C5095" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="D5095" t="n">
         <v>201</v>
@@ -92154,7 +92154,7 @@
         </is>
       </c>
       <c r="C5096" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D5096" t="n">
         <v>201</v>
@@ -92172,7 +92172,7 @@
         </is>
       </c>
       <c r="C5097" t="n">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="D5097" t="n">
         <v>201</v>
@@ -92181,16 +92181,16 @@
     <row r="5098">
       <c r="A5098" t="inlineStr">
         <is>
-          <t>2026/12/31</t>
+          <t>2026/12/30</t>
         </is>
       </c>
       <c r="B5098" t="inlineStr">
         <is>
-          <t>木</t>
+          <t>水</t>
         </is>
       </c>
       <c r="C5098" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D5098" t="n">
         <v>201</v>
@@ -92208,7 +92208,7 @@
         </is>
       </c>
       <c r="C5099" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="D5099" t="n">
         <v>201</v>
@@ -92226,7 +92226,7 @@
         </is>
       </c>
       <c r="C5100" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="D5100" t="n">
         <v>201</v>
@@ -92244,7 +92244,7 @@
         </is>
       </c>
       <c r="C5101" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="D5101" t="n">
         <v>201</v>
@@ -92262,7 +92262,7 @@
         </is>
       </c>
       <c r="C5102" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="D5102" t="n">
         <v>201</v>
@@ -92280,7 +92280,7 @@
         </is>
       </c>
       <c r="C5103" t="n">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="D5103" t="n">
         <v>201</v>
@@ -92289,16 +92289,16 @@
     <row r="5104">
       <c r="A5104" t="inlineStr">
         <is>
-          <t>2027/01/01</t>
+          <t>2026/12/31</t>
         </is>
       </c>
       <c r="B5104" t="inlineStr">
         <is>
-          <t>金</t>
+          <t>木</t>
         </is>
       </c>
       <c r="C5104" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D5104" t="n">
         <v>201</v>
@@ -92316,7 +92316,7 @@
         </is>
       </c>
       <c r="C5105" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D5105" t="n">
         <v>201</v>
@@ -92334,7 +92334,7 @@
         </is>
       </c>
       <c r="C5106" t="n">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="D5106" t="n">
         <v>201</v>
@@ -92352,7 +92352,7 @@
         </is>
       </c>
       <c r="C5107" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D5107" t="n">
         <v>201</v>
@@ -92370,7 +92370,7 @@
         </is>
       </c>
       <c r="C5108" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D5108" t="n">
         <v>201</v>
@@ -92379,16 +92379,16 @@
     <row r="5109">
       <c r="A5109" t="inlineStr">
         <is>
-          <t>2027/01/02</t>
+          <t>2027/01/01</t>
         </is>
       </c>
       <c r="B5109" t="inlineStr">
         <is>
-          <t>土</t>
+          <t>金</t>
         </is>
       </c>
       <c r="C5109" t="n">
-        <v>1</v>
+        <v>19</v>
       </c>
       <c r="D5109" t="n">
         <v>201</v>
@@ -92406,7 +92406,7 @@
         </is>
       </c>
       <c r="C5110" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D5110" t="n">
         <v>201</v>
@@ -92424,7 +92424,7 @@
         </is>
       </c>
       <c r="C5111" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D5111" t="n">
         <v>201</v>
@@ -92442,7 +92442,7 @@
         </is>
       </c>
       <c r="C5112" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="D5112" t="n">
         <v>201</v>
@@ -92460,7 +92460,7 @@
         </is>
       </c>
       <c r="C5113" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D5113" t="n">
         <v>201</v>
@@ -92478,7 +92478,7 @@
         </is>
       </c>
       <c r="C5114" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D5114" t="n">
         <v>201</v>
@@ -92496,7 +92496,7 @@
         </is>
       </c>
       <c r="C5115" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="D5115" t="n">
         <v>201</v>
@@ -92505,16 +92505,16 @@
     <row r="5116">
       <c r="A5116" t="inlineStr">
         <is>
-          <t>2027/01/03</t>
+          <t>2027/01/02</t>
         </is>
       </c>
       <c r="B5116" t="inlineStr">
         <is>
-          <t>日</t>
+          <t>土</t>
         </is>
       </c>
       <c r="C5116" t="n">
-        <v>1</v>
+        <v>22</v>
       </c>
       <c r="D5116" t="n">
         <v>201</v>
@@ -92532,7 +92532,7 @@
         </is>
       </c>
       <c r="C5117" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D5117" t="n">
         <v>201</v>
@@ -92550,7 +92550,7 @@
         </is>
       </c>
       <c r="C5118" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D5118" t="n">
         <v>201</v>
@@ -92568,7 +92568,7 @@
         </is>
       </c>
       <c r="C5119" t="n">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="D5119" t="n">
         <v>201</v>
@@ -92586,7 +92586,7 @@
         </is>
       </c>
       <c r="C5120" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D5120" t="n">
         <v>201</v>
@@ -92604,7 +92604,7 @@
         </is>
       </c>
       <c r="C5121" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D5121" t="n">
         <v>201</v>
@@ -92622,7 +92622,7 @@
         </is>
       </c>
       <c r="C5122" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="D5122" t="n">
         <v>201</v>
@@ -92631,16 +92631,16 @@
     <row r="5123">
       <c r="A5123" t="inlineStr">
         <is>
-          <t>2027/01/04</t>
+          <t>2027/01/03</t>
         </is>
       </c>
       <c r="B5123" t="inlineStr">
         <is>
-          <t>月</t>
+          <t>日</t>
         </is>
       </c>
       <c r="C5123" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D5123" t="n">
         <v>201</v>
@@ -92658,7 +92658,7 @@
         </is>
       </c>
       <c r="C5124" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D5124" t="n">
         <v>201</v>
@@ -92676,7 +92676,7 @@
         </is>
       </c>
       <c r="C5125" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D5125" t="n">
         <v>201</v>
@@ -92694,7 +92694,7 @@
         </is>
       </c>
       <c r="C5126" t="n">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="D5126" t="n">
         <v>201</v>
@@ -92712,7 +92712,7 @@
         </is>
       </c>
       <c r="C5127" t="n">
-        <v>22</v>
+        <v>13</v>
       </c>
       <c r="D5127" t="n">
         <v>201</v>
@@ -92721,16 +92721,16 @@
     <row r="5128">
       <c r="A5128" t="inlineStr">
         <is>
-          <t>2027/01/05</t>
+          <t>2027/01/04</t>
         </is>
       </c>
       <c r="B5128" t="inlineStr">
         <is>
-          <t>火</t>
+          <t>月</t>
         </is>
       </c>
       <c r="C5128" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D5128" t="n">
         <v>201</v>
@@ -92748,9 +92748,27 @@
         </is>
       </c>
       <c r="C5129" t="n">
+        <v>2</v>
+      </c>
+      <c r="D5129" t="n">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="5130">
+      <c r="A5130" t="inlineStr">
+        <is>
+          <t>2027/01/05</t>
+        </is>
+      </c>
+      <c r="B5130" t="inlineStr">
+        <is>
+          <t>火</t>
+        </is>
+      </c>
+      <c r="C5130" t="n">
         <v>7</v>
       </c>
-      <c r="D5129" t="n">
+      <c r="D5130" t="n">
         <v>201</v>
       </c>
     </row>

</xml_diff>

<commit_message>
daily auto push: 2026-10-13 19:50 UTC
</commit_message>
<xml_diff>
--- a/excel/apple2.xlsx
+++ b/excel/apple2.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D5208"/>
+  <dimension ref="A1:D5209"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -93423,16 +93423,16 @@
     <row r="5167">
       <c r="A5167" t="inlineStr">
         <is>
-          <t>2026/12/29</t>
+          <t>2026/10/14</t>
         </is>
       </c>
       <c r="B5167" t="inlineStr">
         <is>
-          <t>火</t>
+          <t>水</t>
         </is>
       </c>
       <c r="C5167" t="n">
-        <v>13</v>
+        <v>2</v>
       </c>
       <c r="D5167" t="n">
         <v>201</v>
@@ -93450,7 +93450,7 @@
         </is>
       </c>
       <c r="C5168" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D5168" t="n">
         <v>201</v>
@@ -93468,7 +93468,7 @@
         </is>
       </c>
       <c r="C5169" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D5169" t="n">
         <v>201</v>
@@ -93486,7 +93486,7 @@
         </is>
       </c>
       <c r="C5170" t="n">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="D5170" t="n">
         <v>201</v>
@@ -93495,16 +93495,16 @@
     <row r="5171">
       <c r="A5171" t="inlineStr">
         <is>
-          <t>2026/12/30</t>
+          <t>2026/12/29</t>
         </is>
       </c>
       <c r="B5171" t="inlineStr">
         <is>
-          <t>水</t>
+          <t>火</t>
         </is>
       </c>
       <c r="C5171" t="n">
-        <v>2</v>
+        <v>23</v>
       </c>
       <c r="D5171" t="n">
         <v>201</v>
@@ -93522,7 +93522,7 @@
         </is>
       </c>
       <c r="C5172" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D5172" t="n">
         <v>201</v>
@@ -93540,7 +93540,7 @@
         </is>
       </c>
       <c r="C5173" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D5173" t="n">
         <v>201</v>
@@ -93558,7 +93558,7 @@
         </is>
       </c>
       <c r="C5174" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="D5174" t="n">
         <v>201</v>
@@ -93576,7 +93576,7 @@
         </is>
       </c>
       <c r="C5175" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D5175" t="n">
         <v>201</v>
@@ -93594,7 +93594,7 @@
         </is>
       </c>
       <c r="C5176" t="n">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="D5176" t="n">
         <v>201</v>
@@ -93603,16 +93603,16 @@
     <row r="5177">
       <c r="A5177" t="inlineStr">
         <is>
-          <t>2026/12/31</t>
+          <t>2026/12/30</t>
         </is>
       </c>
       <c r="B5177" t="inlineStr">
         <is>
-          <t>木</t>
+          <t>水</t>
         </is>
       </c>
       <c r="C5177" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D5177" t="n">
         <v>201</v>
@@ -93630,7 +93630,7 @@
         </is>
       </c>
       <c r="C5178" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="D5178" t="n">
         <v>201</v>
@@ -93648,7 +93648,7 @@
         </is>
       </c>
       <c r="C5179" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="D5179" t="n">
         <v>201</v>
@@ -93666,7 +93666,7 @@
         </is>
       </c>
       <c r="C5180" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="D5180" t="n">
         <v>201</v>
@@ -93684,7 +93684,7 @@
         </is>
       </c>
       <c r="C5181" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="D5181" t="n">
         <v>201</v>
@@ -93702,7 +93702,7 @@
         </is>
       </c>
       <c r="C5182" t="n">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="D5182" t="n">
         <v>201</v>
@@ -93711,16 +93711,16 @@
     <row r="5183">
       <c r="A5183" t="inlineStr">
         <is>
-          <t>2027/01/01</t>
+          <t>2026/12/31</t>
         </is>
       </c>
       <c r="B5183" t="inlineStr">
         <is>
-          <t>金</t>
+          <t>木</t>
         </is>
       </c>
       <c r="C5183" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D5183" t="n">
         <v>201</v>
@@ -93738,7 +93738,7 @@
         </is>
       </c>
       <c r="C5184" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D5184" t="n">
         <v>201</v>
@@ -93756,7 +93756,7 @@
         </is>
       </c>
       <c r="C5185" t="n">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="D5185" t="n">
         <v>201</v>
@@ -93774,7 +93774,7 @@
         </is>
       </c>
       <c r="C5186" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D5186" t="n">
         <v>201</v>
@@ -93792,7 +93792,7 @@
         </is>
       </c>
       <c r="C5187" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D5187" t="n">
         <v>201</v>
@@ -93801,16 +93801,16 @@
     <row r="5188">
       <c r="A5188" t="inlineStr">
         <is>
-          <t>2027/01/02</t>
+          <t>2027/01/01</t>
         </is>
       </c>
       <c r="B5188" t="inlineStr">
         <is>
-          <t>土</t>
+          <t>金</t>
         </is>
       </c>
       <c r="C5188" t="n">
-        <v>1</v>
+        <v>19</v>
       </c>
       <c r="D5188" t="n">
         <v>201</v>
@@ -93828,7 +93828,7 @@
         </is>
       </c>
       <c r="C5189" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D5189" t="n">
         <v>201</v>
@@ -93846,7 +93846,7 @@
         </is>
       </c>
       <c r="C5190" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D5190" t="n">
         <v>201</v>
@@ -93864,7 +93864,7 @@
         </is>
       </c>
       <c r="C5191" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="D5191" t="n">
         <v>201</v>
@@ -93882,7 +93882,7 @@
         </is>
       </c>
       <c r="C5192" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D5192" t="n">
         <v>201</v>
@@ -93900,7 +93900,7 @@
         </is>
       </c>
       <c r="C5193" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D5193" t="n">
         <v>201</v>
@@ -93918,7 +93918,7 @@
         </is>
       </c>
       <c r="C5194" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="D5194" t="n">
         <v>201</v>
@@ -93927,16 +93927,16 @@
     <row r="5195">
       <c r="A5195" t="inlineStr">
         <is>
-          <t>2027/01/03</t>
+          <t>2027/01/02</t>
         </is>
       </c>
       <c r="B5195" t="inlineStr">
         <is>
-          <t>日</t>
+          <t>土</t>
         </is>
       </c>
       <c r="C5195" t="n">
-        <v>1</v>
+        <v>22</v>
       </c>
       <c r="D5195" t="n">
         <v>201</v>
@@ -93954,7 +93954,7 @@
         </is>
       </c>
       <c r="C5196" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D5196" t="n">
         <v>201</v>
@@ -93972,7 +93972,7 @@
         </is>
       </c>
       <c r="C5197" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D5197" t="n">
         <v>201</v>
@@ -93990,7 +93990,7 @@
         </is>
       </c>
       <c r="C5198" t="n">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="D5198" t="n">
         <v>201</v>
@@ -94008,7 +94008,7 @@
         </is>
       </c>
       <c r="C5199" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D5199" t="n">
         <v>201</v>
@@ -94026,7 +94026,7 @@
         </is>
       </c>
       <c r="C5200" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D5200" t="n">
         <v>201</v>
@@ -94044,7 +94044,7 @@
         </is>
       </c>
       <c r="C5201" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="D5201" t="n">
         <v>201</v>
@@ -94053,16 +94053,16 @@
     <row r="5202">
       <c r="A5202" t="inlineStr">
         <is>
-          <t>2027/01/04</t>
+          <t>2027/01/03</t>
         </is>
       </c>
       <c r="B5202" t="inlineStr">
         <is>
-          <t>月</t>
+          <t>日</t>
         </is>
       </c>
       <c r="C5202" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D5202" t="n">
         <v>201</v>
@@ -94080,7 +94080,7 @@
         </is>
       </c>
       <c r="C5203" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D5203" t="n">
         <v>201</v>
@@ -94098,7 +94098,7 @@
         </is>
       </c>
       <c r="C5204" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D5204" t="n">
         <v>201</v>
@@ -94116,7 +94116,7 @@
         </is>
       </c>
       <c r="C5205" t="n">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="D5205" t="n">
         <v>201</v>
@@ -94134,7 +94134,7 @@
         </is>
       </c>
       <c r="C5206" t="n">
-        <v>22</v>
+        <v>13</v>
       </c>
       <c r="D5206" t="n">
         <v>201</v>
@@ -94143,16 +94143,16 @@
     <row r="5207">
       <c r="A5207" t="inlineStr">
         <is>
-          <t>2027/01/05</t>
+          <t>2027/01/04</t>
         </is>
       </c>
       <c r="B5207" t="inlineStr">
         <is>
-          <t>火</t>
+          <t>月</t>
         </is>
       </c>
       <c r="C5207" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D5207" t="n">
         <v>201</v>
@@ -94170,9 +94170,27 @@
         </is>
       </c>
       <c r="C5208" t="n">
+        <v>2</v>
+      </c>
+      <c r="D5208" t="n">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="5209">
+      <c r="A5209" t="inlineStr">
+        <is>
+          <t>2027/01/05</t>
+        </is>
+      </c>
+      <c r="B5209" t="inlineStr">
+        <is>
+          <t>火</t>
+        </is>
+      </c>
+      <c r="C5209" t="n">
         <v>7</v>
       </c>
-      <c r="D5208" t="n">
+      <c r="D5209" t="n">
         <v>201</v>
       </c>
     </row>

</xml_diff>

<commit_message>
daily auto push: 2026-10-29 16:01 UTC
</commit_message>
<xml_diff>
--- a/excel/apple2.xlsx
+++ b/excel/apple2.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D5318"/>
+  <dimension ref="A1:D5319"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -95403,16 +95403,16 @@
     <row r="5277">
       <c r="A5277" t="inlineStr">
         <is>
-          <t>2026/12/29</t>
+          <t>2026/10/30</t>
         </is>
       </c>
       <c r="B5277" t="inlineStr">
         <is>
-          <t>火</t>
+          <t>金</t>
         </is>
       </c>
       <c r="C5277" t="n">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="D5277" t="n">
         <v>201</v>
@@ -95430,7 +95430,7 @@
         </is>
       </c>
       <c r="C5278" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D5278" t="n">
         <v>201</v>
@@ -95448,7 +95448,7 @@
         </is>
       </c>
       <c r="C5279" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D5279" t="n">
         <v>201</v>
@@ -95466,7 +95466,7 @@
         </is>
       </c>
       <c r="C5280" t="n">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="D5280" t="n">
         <v>201</v>
@@ -95475,16 +95475,16 @@
     <row r="5281">
       <c r="A5281" t="inlineStr">
         <is>
-          <t>2026/12/30</t>
+          <t>2026/12/29</t>
         </is>
       </c>
       <c r="B5281" t="inlineStr">
         <is>
-          <t>水</t>
+          <t>火</t>
         </is>
       </c>
       <c r="C5281" t="n">
-        <v>2</v>
+        <v>23</v>
       </c>
       <c r="D5281" t="n">
         <v>201</v>
@@ -95502,7 +95502,7 @@
         </is>
       </c>
       <c r="C5282" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D5282" t="n">
         <v>201</v>
@@ -95520,7 +95520,7 @@
         </is>
       </c>
       <c r="C5283" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D5283" t="n">
         <v>201</v>
@@ -95538,7 +95538,7 @@
         </is>
       </c>
       <c r="C5284" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="D5284" t="n">
         <v>201</v>
@@ -95556,7 +95556,7 @@
         </is>
       </c>
       <c r="C5285" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D5285" t="n">
         <v>201</v>
@@ -95574,7 +95574,7 @@
         </is>
       </c>
       <c r="C5286" t="n">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="D5286" t="n">
         <v>201</v>
@@ -95583,16 +95583,16 @@
     <row r="5287">
       <c r="A5287" t="inlineStr">
         <is>
-          <t>2026/12/31</t>
+          <t>2026/12/30</t>
         </is>
       </c>
       <c r="B5287" t="inlineStr">
         <is>
-          <t>木</t>
+          <t>水</t>
         </is>
       </c>
       <c r="C5287" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D5287" t="n">
         <v>201</v>
@@ -95610,7 +95610,7 @@
         </is>
       </c>
       <c r="C5288" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="D5288" t="n">
         <v>201</v>
@@ -95628,7 +95628,7 @@
         </is>
       </c>
       <c r="C5289" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="D5289" t="n">
         <v>201</v>
@@ -95646,7 +95646,7 @@
         </is>
       </c>
       <c r="C5290" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="D5290" t="n">
         <v>201</v>
@@ -95664,7 +95664,7 @@
         </is>
       </c>
       <c r="C5291" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="D5291" t="n">
         <v>201</v>
@@ -95682,7 +95682,7 @@
         </is>
       </c>
       <c r="C5292" t="n">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="D5292" t="n">
         <v>201</v>
@@ -95691,16 +95691,16 @@
     <row r="5293">
       <c r="A5293" t="inlineStr">
         <is>
-          <t>2027/01/01</t>
+          <t>2026/12/31</t>
         </is>
       </c>
       <c r="B5293" t="inlineStr">
         <is>
-          <t>金</t>
+          <t>木</t>
         </is>
       </c>
       <c r="C5293" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D5293" t="n">
         <v>201</v>
@@ -95718,7 +95718,7 @@
         </is>
       </c>
       <c r="C5294" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D5294" t="n">
         <v>201</v>
@@ -95736,7 +95736,7 @@
         </is>
       </c>
       <c r="C5295" t="n">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="D5295" t="n">
         <v>201</v>
@@ -95754,7 +95754,7 @@
         </is>
       </c>
       <c r="C5296" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D5296" t="n">
         <v>201</v>
@@ -95772,7 +95772,7 @@
         </is>
       </c>
       <c r="C5297" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D5297" t="n">
         <v>201</v>
@@ -95781,16 +95781,16 @@
     <row r="5298">
       <c r="A5298" t="inlineStr">
         <is>
-          <t>2027/01/02</t>
+          <t>2027/01/01</t>
         </is>
       </c>
       <c r="B5298" t="inlineStr">
         <is>
-          <t>土</t>
+          <t>金</t>
         </is>
       </c>
       <c r="C5298" t="n">
-        <v>1</v>
+        <v>19</v>
       </c>
       <c r="D5298" t="n">
         <v>201</v>
@@ -95808,7 +95808,7 @@
         </is>
       </c>
       <c r="C5299" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D5299" t="n">
         <v>201</v>
@@ -95826,7 +95826,7 @@
         </is>
       </c>
       <c r="C5300" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D5300" t="n">
         <v>201</v>
@@ -95844,7 +95844,7 @@
         </is>
       </c>
       <c r="C5301" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="D5301" t="n">
         <v>201</v>
@@ -95862,7 +95862,7 @@
         </is>
       </c>
       <c r="C5302" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D5302" t="n">
         <v>201</v>
@@ -95880,7 +95880,7 @@
         </is>
       </c>
       <c r="C5303" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D5303" t="n">
         <v>201</v>
@@ -95898,7 +95898,7 @@
         </is>
       </c>
       <c r="C5304" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="D5304" t="n">
         <v>201</v>
@@ -95907,16 +95907,16 @@
     <row r="5305">
       <c r="A5305" t="inlineStr">
         <is>
-          <t>2027/01/03</t>
+          <t>2027/01/02</t>
         </is>
       </c>
       <c r="B5305" t="inlineStr">
         <is>
-          <t>日</t>
+          <t>土</t>
         </is>
       </c>
       <c r="C5305" t="n">
-        <v>1</v>
+        <v>22</v>
       </c>
       <c r="D5305" t="n">
         <v>201</v>
@@ -95934,7 +95934,7 @@
         </is>
       </c>
       <c r="C5306" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D5306" t="n">
         <v>201</v>
@@ -95952,7 +95952,7 @@
         </is>
       </c>
       <c r="C5307" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D5307" t="n">
         <v>201</v>
@@ -95970,7 +95970,7 @@
         </is>
       </c>
       <c r="C5308" t="n">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="D5308" t="n">
         <v>201</v>
@@ -95988,7 +95988,7 @@
         </is>
       </c>
       <c r="C5309" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D5309" t="n">
         <v>201</v>
@@ -96006,7 +96006,7 @@
         </is>
       </c>
       <c r="C5310" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D5310" t="n">
         <v>201</v>
@@ -96024,7 +96024,7 @@
         </is>
       </c>
       <c r="C5311" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="D5311" t="n">
         <v>201</v>
@@ -96033,16 +96033,16 @@
     <row r="5312">
       <c r="A5312" t="inlineStr">
         <is>
-          <t>2027/01/04</t>
+          <t>2027/01/03</t>
         </is>
       </c>
       <c r="B5312" t="inlineStr">
         <is>
-          <t>月</t>
+          <t>日</t>
         </is>
       </c>
       <c r="C5312" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D5312" t="n">
         <v>201</v>
@@ -96060,7 +96060,7 @@
         </is>
       </c>
       <c r="C5313" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D5313" t="n">
         <v>201</v>
@@ -96078,7 +96078,7 @@
         </is>
       </c>
       <c r="C5314" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D5314" t="n">
         <v>201</v>
@@ -96096,7 +96096,7 @@
         </is>
       </c>
       <c r="C5315" t="n">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="D5315" t="n">
         <v>201</v>
@@ -96114,7 +96114,7 @@
         </is>
       </c>
       <c r="C5316" t="n">
-        <v>22</v>
+        <v>13</v>
       </c>
       <c r="D5316" t="n">
         <v>201</v>
@@ -96123,16 +96123,16 @@
     <row r="5317">
       <c r="A5317" t="inlineStr">
         <is>
-          <t>2027/01/05</t>
+          <t>2027/01/04</t>
         </is>
       </c>
       <c r="B5317" t="inlineStr">
         <is>
-          <t>火</t>
+          <t>月</t>
         </is>
       </c>
       <c r="C5317" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D5317" t="n">
         <v>201</v>
@@ -96150,9 +96150,27 @@
         </is>
       </c>
       <c r="C5318" t="n">
+        <v>2</v>
+      </c>
+      <c r="D5318" t="n">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="5319">
+      <c r="A5319" t="inlineStr">
+        <is>
+          <t>2027/01/05</t>
+        </is>
+      </c>
+      <c r="B5319" t="inlineStr">
+        <is>
+          <t>火</t>
+        </is>
+      </c>
+      <c r="C5319" t="n">
         <v>7</v>
       </c>
-      <c r="D5318" t="n">
+      <c r="D5319" t="n">
         <v>201</v>
       </c>
     </row>

</xml_diff>